<commit_message>
feat: apply definitive balance mod suite across all game binaries
apply definitive balance mod suite across all game binaries, tables, and
Euthys school lessons
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/equipment.xlsx
+++ b/mod_project/data_tables/equipment.xlsx
@@ -510,7 +510,7 @@
       <c r="F2" t="inlineStr">
         <is>
           <t>One-handed sword that's easy to handle.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 0]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 0]
 Innate: Standard equipment without innate passive enchantments.</t>
         </is>
       </c>
@@ -547,7 +547,7 @@
       <c r="F3" t="inlineStr">
         <is>
           <t>One-handed sword with some weight and a thicker edge.
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 0]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 0]
 Innate: Standard equipment without innate passive enchantments.</t>
         </is>
       </c>
@@ -584,7 +584,7 @@
       <c r="F4" t="inlineStr">
         <is>
           <t>Terrible at cutting, but weirdly easy to land hits with.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 2]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 2]
 Innate: Phys Hit +10% | Phys Hit +5%</t>
         </is>
       </c>
@@ -621,7 +621,7 @@
       <c r="F5" t="inlineStr">
         <is>
           <t>Every journey starts with this weapon!
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 2]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 2]
 Innate: Crit Rate +10% | Action Speed +5%</t>
         </is>
       </c>
@@ -658,7 +658,7 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>Super effective towards feline types. It's cat-astrophic!
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 1]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 1]
 Innate: Physical ATK vs. Felines +100%</t>
         </is>
       </c>
@@ -695,7 +695,7 @@
       <c r="F7" t="inlineStr">
         <is>
           <t>Magic sword passed down in the royal family. More versatile now.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 4]
 Innate: Max HP +5% | Max TP +5% | Phys ATK +10% | Magic ATK +10%</t>
         </is>
       </c>
@@ -732,7 +732,7 @@
       <c r="F8" t="inlineStr">
         <is>
           <t>Frightening sword that sends its wielder to the world of lilies.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 4]
 Innate: Wind Magic +15% | Phys Dodge +10% | Magic Dodge +10% | Action Speed +10%</t>
         </is>
       </c>
@@ -769,7 +769,7 @@
       <c r="F9" t="inlineStr">
         <is>
           <t>Sword of a maiden who sacrificed her future to liberate her homeland.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 4]
 Innate: Normal attacks: 10% TP Drain | RES +10% | AGI +10% | Fire Res -40</t>
         </is>
       </c>
@@ -806,7 +806,7 @@
       <c r="F10" t="inlineStr">
         <is>
           <t>Yanked out from inside a holy tree. Purifies its wielder's soul.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 4]
 Innate: Max TP +10% | HP Regen +4%/turn | TP Regen +4/turn</t>
         </is>
       </c>
@@ -843,7 +843,7 @@
       <c r="F11" t="inlineStr">
         <is>
           <t>This quickly oscillating blade can cut anything it touches in two.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 4]
 Innate: DEX +10% | Phys Hit +10% | Phys Dodge +10% | Crit Rate +10%</t>
         </is>
       </c>
@@ -880,7 +880,7 @@
       <c r="F12" t="inlineStr">
         <is>
           <t>Black sword of the king of the elves. Capable of slaying gods.
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 4]
 Innate: Physical ATK vs. Magic Beings +100% | Phys DEF +10% | Magic Dodge +10%</t>
         </is>
       </c>
@@ -917,7 +917,7 @@
       <c r="F13" t="inlineStr">
         <is>
           <t>Treasured sword enveloped in flames that burn down evil.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 4]
 Innate: Fire Magic +15% | Physical ATK vs. Apparitions +50% | DEX +10%</t>
         </is>
       </c>
@@ -954,7 +954,7 @@
       <c r="F14" t="inlineStr">
         <is>
           <t>Purifying sword that was owned by one of God's 12 servant spirits.
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 4]
 Innate: Physical ATK vs. Humans +100% | Action Speed +10% | Damage -&gt; TP (10%)</t>
         </is>
       </c>
@@ -991,7 +991,7 @@
       <c r="F15" t="inlineStr">
         <is>
           <t>Dragonslaying sword, ten hands long.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 4]
 Innate: Physical ATK vs. Dragons +100% | Phys Hit +10% | Water Res +50 | Nullify stun</t>
         </is>
       </c>
@@ -1028,7 +1028,7 @@
       <c r="F16" t="inlineStr">
         <is>
           <t>The demon king's favorite red sword.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 4]
 Innate: Physical ATK vs. Demons +100% | Magic ATK +10% | Chant Speed +15%</t>
         </is>
       </c>
@@ -1065,7 +1065,7 @@
       <c r="F17" t="inlineStr">
         <is>
           <t>Sword that stores evil power by absorbing the life of others.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 4]
 Innate: Physical ATK vs. Demons +50% | Physical ATK vs. Humans +50%</t>
         </is>
       </c>
@@ -1102,7 +1102,7 @@
       <c r="F18" t="inlineStr">
         <is>
           <t>Sword that has stored dragon and tiger spirits for a millennium.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 4]
 Innate: Physical ATK vs. Undead +100% | DEX +10% | AGI +10%</t>
         </is>
       </c>
@@ -1139,7 +1139,7 @@
       <c r="F19" t="inlineStr">
         <is>
           <t>Heavy two-handed sword that can only be handled by swordsmen.
-[Weapon | Range: Short | Delay: E+ (2.45x) | Slots: 0]
+[Weapon | Range: Short | Delay: E+ (2.05x) | Slots: 0]
 Innate: Standard equipment without innate passive enchantments.</t>
         </is>
       </c>
@@ -1176,7 +1176,7 @@
       <c r="F20" t="inlineStr">
         <is>
           <t>Short for a two-handed sword. Easy to handle and great for beginners.
-[Weapon | Range: Short | Delay: E+ (2.45x) | Slots: 2]
+[Weapon | Range: Short | Delay: E+ (2.05x) | Slots: 2]
 Innate: DEF +5% | Action Speed +5%</t>
         </is>
       </c>
@@ -1213,7 +1213,7 @@
       <c r="F21" t="inlineStr">
         <is>
           <t>Big, long sword for competing with lances. Who's inadequate now?
-[Weapon | Range: Short | Delay: D (2.3x) | Slots: 3]
+[Weapon | Range: Short | Delay: D (1.95x) | Slots: 3]
 Innate: AGI +5% | Aggro/Enmity +25%</t>
         </is>
       </c>
@@ -1250,7 +1250,7 @@
       <c r="F22" t="inlineStr">
         <is>
           <t>Holy sword made to hunt down the impure undead.
-[Weapon | Range: Short | Delay: D+ (2.15x) | Slots: 3]
+[Weapon | Range: Short | Delay: D+ (1.85x) | Slots: 3]
 Innate: Physical ATK vs. Undead +20% | DEF +10% | DEX +10%</t>
         </is>
       </c>
@@ -1287,7 +1287,7 @@
       <c r="F23" t="inlineStr">
         <is>
           <t>Sword with a tuning fork on the pommel. Enhances your singing.
-[Weapon | Range: Short | Delay: D+ (2.15x) | Slots: 4]
+[Weapon | Range: Short | Delay: D+ (1.85x) | Slots: 4]
 Innate: Physical ATK vs. Sea Creatures +100% | Song Potency +20% (Carol/Chorale etc.)</t>
         </is>
       </c>
@@ -1324,7 +1324,7 @@
       <c r="F24" t="inlineStr">
         <is>
           <t>Too big, thick, heavy, and long for a sword. This is a slab of iron.
-[Weapon | Range: Short | Delay: F+ (2.75x) | Slots: 3]
+[Weapon | Range: Short | Delay: F+ (2.25x) | Slots: 3]
 Innate: Physical ATK vs. Demons +50% | Physical ATK vs. Undead +50% | DEF +10%</t>
         </is>
       </c>
@@ -1361,7 +1361,7 @@
       <c r="F25" t="inlineStr">
         <is>
           <t>Magic sword that can penetrate any armor.
-[Weapon | Range: Short | Delay: D+ (2.15x) | Slots: 4]
+[Weapon | Range: Short | Delay: D+ (1.85x) | Slots: 4]
 Innate: Physical ATK vs. Humans +20% | INT +10% | Phys Hit +10% | TP Regen +2/turn</t>
         </is>
       </c>
@@ -1398,7 +1398,7 @@
       <c r="F26" t="inlineStr">
         <is>
           <t>Sword for a more famous member of the Knights of the Round Table.
-[Weapon | Range: Short | Delay: E+ (2.45x) | Slots: 4]
+[Weapon | Range: Short | Delay: E+ (2.05x) | Slots: 4]
 Innate: Normal attacks: Silence chance (20%) | DEF +10% | Crit Rate +10%</t>
         </is>
       </c>
@@ -1435,7 +1435,7 @@
       <c r="F27" t="inlineStr">
         <is>
           <t>Iconic royal family sword, upgraded so much that it now takes two hands.
-[Weapon | Range: Short | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Short | Delay: D (1.95x) | Slots: 4]
 Innate: Max TP +10% | Phys ATK +10% | Magic ATK +10%</t>
         </is>
       </c>
@@ -1472,7 +1472,7 @@
       <c r="F28" t="inlineStr">
         <is>
           <t>Sword of anger that cuts through everything. Slayer of dragons.
-[Weapon | Range: Short | Delay: E+ (2.45x) | Slots: 4]
+[Weapon | Range: Short | Delay: E+ (2.05x) | Slots: 4]
 Innate: Physical ATK vs. Dragons +50% | DEF +5% | RES +5% | AGI +10%</t>
         </is>
       </c>
@@ -1509,7 +1509,7 @@
       <c r="F29" t="inlineStr">
         <is>
           <t>Turns any situation into a beneficial one for you. Kinda cheat-y.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 4]
 Innate: Pep is fixed at the max value | Damage -&gt; TP (10%) | Damage -&gt; TP (10%)</t>
         </is>
       </c>
@@ -1546,7 +1546,7 @@
       <c r="F30" t="inlineStr">
         <is>
           <t>Holy sword from a woman lying in a pond. Came with a magic scabbard.
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 4]
 Innate: Water Magic +15% | Water Res +50 | HP Regen +8%/turn</t>
         </is>
       </c>
@@ -1583,7 +1583,7 @@
       <c r="F31" t="inlineStr">
         <is>
           <t>Sword with an illuminating blade made of magic.
-[Weapon | Range: Short | Delay: D+ (2.15x) | Slots: 4]
+[Weapon | Range: Short | Delay: D+ (1.85x) | Slots: 4]
 Innate: Physical ATK vs. Undead +50% | Max TP +10% | DEF +10% | Crit Rate +10%</t>
         </is>
       </c>
@@ -1620,7 +1620,7 @@
       <c r="F32" t="inlineStr">
         <is>
           <t>Legendary sword that holds both light and dark.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 4]
 Innate: Physical ATK vs. Demons +50% | Action Speed +10% | Chant Speed +15%</t>
         </is>
       </c>
@@ -1657,7 +1657,7 @@
       <c r="F33" t="inlineStr">
         <is>
           <t>Sword that was owned by the flame giant. Burns through everything.
-[Weapon | Range: Short | Delay: E+ (2.45x) | Slots: 4]
+[Weapon | Range: Short | Delay: E+ (2.05x) | Slots: 4]
 Innate: Fire Magic +15% | Normal attacks: Paralysis chance (20%) | HP Regen +4%/turn</t>
         </is>
       </c>
@@ -1694,7 +1694,7 @@
       <c r="F34" t="inlineStr">
         <is>
           <t>Wielding this sword allows you to vanquish anything.
-[Weapon | Range: Short | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Short | Delay: D (1.95x) | Slots: 4]
 Innate: Physical ATK vs. Dragons +50% | Normal attacks: 20% TP Drain</t>
         </is>
       </c>
@@ -1731,7 +1731,7 @@
       <c r="F35" t="inlineStr">
         <is>
           <t>Double-edged knife that stabs the enemy.
-[Weapon | Range: Short | Delay: A (1.2x) | Slots: 0]
+[Weapon | Range: Short | Delay: A (1.15x) | Slots: 0]
 Innate: Standard equipment without innate passive enchantments.</t>
         </is>
       </c>
@@ -1768,7 +1768,7 @@
       <c r="F36" t="inlineStr">
         <is>
           <t>Knife that leaves the fruit world trembling in fear.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 2]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 2]
 Innate: Physical ATK vs. Fruit +50% | Crit Rate +10%</t>
         </is>
       </c>
@@ -1805,7 +1805,7 @@
       <c r="F37" t="inlineStr">
         <is>
           <t>Fish and fishfolk shudder at the very sight of it.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 2]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 2]
 Innate: Physical ATK vs. Sea Creatures +100% | Phys Hit +10%</t>
         </is>
       </c>
@@ -1842,7 +1842,7 @@
       <c r="F38" t="inlineStr">
         <is>
           <t>Double-edged knife used in the Renaissance era.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 3]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 3]
 Innate: Max HP +5% | Max TP +10% | Action Speed +5%</t>
         </is>
       </c>
@@ -1879,7 +1879,7 @@
       <c r="F39" t="inlineStr">
         <is>
           <t>Magic dagger for purposes both ceremonial and stabby.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 3]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 3]
 Innate: Max TP +10% | Interrupt Rate -50% | Magic Damage Taken -10%</t>
         </is>
       </c>
@@ -1916,7 +1916,7 @@
       <c r="F40" t="inlineStr">
         <is>
           <t>A pocket-sized, easy-to-wield dagger used by assassins.
-[Weapon | Range: Short | Delay: A (1.2x) | Slots: 3]
+[Weapon | Range: Short | Delay: A (1.15x) | Slots: 3]
 Innate: Normal attacks: Instakill chance (15%) | AGI +10% | Phys Hit +10%</t>
         </is>
       </c>
@@ -1953,7 +1953,7 @@
       <c r="F41" t="inlineStr">
         <is>
           <t>Blood-seeking knife of darkness.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 4]
 Innate: Normal attacks: 20% HP Drain | Max TP +10% | Aggro/Enmity -25%</t>
         </is>
       </c>
@@ -1990,7 +1990,7 @@
       <c r="F42" t="inlineStr">
         <is>
           <t>Specialized knife for the slaying of sorcerers.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 4]
 Innate: Normal attacks: 20% TP Drain | Magic DEF +10% | Magic DEF +10%</t>
         </is>
       </c>
@@ -2027,7 +2027,7 @@
       <c r="F43" t="inlineStr">
         <is>
           <t>Knife that looks like a miniature sickle.
-[Weapon | Range: Short | Delay: A (1.2x) | Slots: 4]
+[Weapon | Range: Short | Delay: A (1.15x) | Slots: 4]
 Innate: Normal attacks: Paralysis chance (20%) | RES +10% | Action Speed +10%</t>
         </is>
       </c>
@@ -2064,7 +2064,7 @@
       <c r="F44" t="inlineStr">
         <is>
           <t>Kitchen knife used by someone aiming to be the god of cookery.
-[Weapon | Range: Short | Delay: A (1.2x) | Slots: 3]
+[Weapon | Range: Short | Delay: A (1.15x) | Slots: 3]
 Innate: Physical ATK vs. Fruit +100% | Physical ATK vs. Sea Creatures +100%</t>
         </is>
       </c>
@@ -2101,7 +2101,7 @@
       <c r="F45" t="inlineStr">
         <is>
           <t>Knife forged by alchemy. In the jewel on its pommel, a demon is sealed.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 4]
 Innate: Max TP +10% | Magic ATK +10% | Magic Damage Taken -10% | TP Regen +4/turn</t>
         </is>
       </c>
@@ -2138,7 +2138,7 @@
       <c r="F46" t="inlineStr">
         <is>
           <t>Personal protection weapon of a god of blacksmithing.
-[Weapon | Range: Short | Delay: A (1.2x) | Slots: 4]
+[Weapon | Range: Short | Delay: A (1.15x) | Slots: 4]
 Innate: Fire Magic +15% | DEX +10% | AGI +10% | All Phys Res +15</t>
         </is>
       </c>
@@ -2175,7 +2175,7 @@
       <c r="F47" t="inlineStr">
         <is>
           <t>Sacred Jamadhar wielded by the king of battles.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 4]
 Innate: Phys Dodge +10% | Nullify stun</t>
         </is>
       </c>
@@ -2212,7 +2212,7 @@
       <c r="F48" t="inlineStr">
         <is>
           <t>Spoke of a wheel that drives evildoers to hell.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 4]
 Innate: Physical ATK vs. Humans +100% | Normal attacks: Instakill chance (15%)</t>
         </is>
       </c>
@@ -2249,7 +2249,7 @@
       <c r="F49" t="inlineStr">
         <is>
           <t>Knife with a moral compass. Stab someone nice and they won't even feel it.
-[Weapon | Range: Short | Delay: A (1.2x) | Slots: 4]
+[Weapon | Range: Short | Delay: A (1.15x) | Slots: 4]
 Innate: Max TP +10% | Phys ATK +10% | Earth Res +50</t>
         </is>
       </c>
@@ -2286,7 +2286,7 @@
       <c r="F50" t="inlineStr">
         <is>
           <t>Dagger filled with hate by the dark god who bides beneath the abyss.
-[Weapon | Range: Short | Delay: A+ (1.0x) | Slots: 4]
+[Weapon | Range: Short | Delay: A+ (1.00x) | Slots: 4]
 Innate: Normal attacks: Slow chance (15%) | Action Speed +10% | Action Speed +10%</t>
         </is>
       </c>
@@ -2323,7 +2323,7 @@
       <c r="F51" t="inlineStr">
         <is>
           <t>Large knife in the shape of an L.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 0]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 0]
 Innate: Standard equipment without innate passive enchantments.</t>
         </is>
       </c>
@@ -2360,7 +2360,7 @@
       <c r="F52" t="inlineStr">
         <is>
           <t>Supple and beautiful cutlery made out of damuscus steel.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 2]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 2]
 Innate: Phys Hit +10% | Crit Rate +5%</t>
         </is>
       </c>
@@ -2397,7 +2397,7 @@
       <c r="F53" t="inlineStr">
         <is>
           <t>Large knife with a curved edge.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 2]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 2]
 Innate: DEX +10% | AGI +5%</t>
         </is>
       </c>
@@ -2434,7 +2434,7 @@
       <c r="F54" t="inlineStr">
         <is>
           <t>Wide, long, heavy dagger that can cut through light armor.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 3]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 3]
 Innate: Phys Hit +10% | Crit Rate +10% | Action Speed +5%</t>
         </is>
       </c>
@@ -2471,7 +2471,7 @@
       <c r="F55" t="inlineStr">
         <is>
           <t>Unique weapon that pirates like to use.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 2]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 2]
 Innate: Physical ATK vs. Sea Creatures +100% | Water Res +50</t>
         </is>
       </c>
@@ -2508,7 +2508,7 @@
       <c r="F56" t="inlineStr">
         <is>
           <t>Punches through gaps in armor to deliver the paralyzing agent on its tip.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 4]
 Innate: Normal attacks: Paralysis chance (20%) | Max HP +5% | Phys Dodge +10%</t>
         </is>
       </c>
@@ -2545,7 +2545,7 @@
       <c r="F57" t="inlineStr">
         <is>
           <t>Named after mistletoe that pierced a god.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 4]
 Innate: Normal attacks: 10% TP Drain | Max TP +10% | Phys Hit +10% | Magic DEF +10%</t>
         </is>
       </c>
@@ -2582,7 +2582,7 @@
       <c r="F58" t="inlineStr">
         <is>
           <t>For the discerning decapitator.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 4]
 Innate: Physical ATK vs. Humans +20% | DEX +10% | Action Speed +10%</t>
         </is>
       </c>
@@ -2619,7 +2619,7 @@
       <c r="F59" t="inlineStr">
         <is>
           <t>S-shaped knife meant to insert and slice through gaps in armor.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 4]
 Innate: Normal attacks: Stun chance (20%) | Phys Dodge +10% | Magic Dodge +10%</t>
         </is>
       </c>
@@ -2656,7 +2656,7 @@
       <c r="F60" t="inlineStr">
         <is>
           <t>Long knife with a poison needle built in. Sharp enough without it.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 3]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 3]
 Innate: Normal attacks: Poison chance (20%) | DEX +10% | Earth Res +50</t>
         </is>
       </c>
@@ -2693,7 +2693,7 @@
       <c r="F61" t="inlineStr">
         <is>
           <t>Wielding this will make you yearn to hurt somebody.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 4]
 Innate: Physical ATK vs. Humans +50% | Normal attacks: 20% HP Drain</t>
         </is>
       </c>
@@ -2730,7 +2730,7 @@
       <c r="F62" t="inlineStr">
         <is>
           <t>Man-eating kukri that chomps at the bit for destruction.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 4]
 Innate: Phys ATK +10% | Phys Hit +10% | Phys Dodge +10% | Crit Rate +10%</t>
         </is>
       </c>
@@ -2767,7 +2767,7 @@
       <c r="F63" t="inlineStr">
         <is>
           <t>Shotel with a blade made out of unknown energy.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 4]
 Innate: Physical ATK vs. Magic Beings +50% | Phys DEF +10% | Slash Res +50</t>
         </is>
       </c>
@@ -2804,7 +2804,7 @@
       <c r="F64" t="inlineStr">
         <is>
           <t>Dagger decorated with a four-leaf clover.
-[Weapon | Range: Short | Delay: A (1.2x) | Slots: 4]
+[Weapon | Range: Short | Delay: A (1.15x) | Slots: 4]
 Innate: AGI +10% | Phys Dodge +10% | Action Speed +10% | All Elem Res +15</t>
         </is>
       </c>
@@ -2841,7 +2841,7 @@
       <c r="F65" t="inlineStr">
         <is>
           <t>It's said that even a tiny cut from this will erase your soul.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 4]
 Innate: Normal attacks: Instakill chance (15%) | AGI +10% | Stab Res +30</t>
         </is>
       </c>
@@ -2878,7 +2878,7 @@
       <c r="F66" t="inlineStr">
         <is>
           <t>Kukri of a war-goddess who stamps gods of destruction underfoot.
-[Weapon | Range: Short | Delay: A (1.2x) | Slots: 4]
+[Weapon | Range: Short | Delay: A (1.15x) | Slots: 4]
 Innate: Normal attacks: Petrify chance (15%) | Physical ATK vs. Demons +100%</t>
         </is>
       </c>
@@ -2915,7 +2915,7 @@
       <c r="F67" t="inlineStr">
         <is>
           <t>Small axe that can be wielded in one hand.
-[Weapon | Range: Short | Delay: D (2.3x) | Slots: 0]
+[Weapon | Range: Short | Delay: D (1.95x) | Slots: 0]
 Innate: Standard equipment without innate passive enchantments.</t>
         </is>
       </c>
@@ -2952,7 +2952,7 @@
       <c r="F68" t="inlineStr">
         <is>
           <t>Small and easy-to-use axe.
-[Weapon | Range: Short | Delay: D+ (2.15x) | Slots: 3]
+[Weapon | Range: Short | Delay: D+ (1.85x) | Slots: 3]
 Innate: DEX +10% | Phys Hit +5% | Aggro/Enmity +25%</t>
         </is>
       </c>
@@ -2989,7 +2989,7 @@
       <c r="F69" t="inlineStr">
         <is>
           <t>Mountain climbing equipment with a nasty surprise.
-[Weapon | Range: Short | Delay: D (2.3x) | Slots: 2]
+[Weapon | Range: Short | Delay: D (1.95x) | Slots: 2]
 Innate: Lightning Magic +15%</t>
         </is>
       </c>
@@ -3026,7 +3026,7 @@
       <c r="F70" t="inlineStr">
         <is>
           <t>The bane of naughty children. This means you, Fried.
-[Weapon | Range: Short | Delay: E+ (2.45x) | Slots: 2]
+[Weapon | Range: Short | Delay: E+ (2.05x) | Slots: 2]
 Innate: Phys Hit +10% | TP Regen +4/turn</t>
         </is>
       </c>
@@ -3063,7 +3063,7 @@
       <c r="F71" t="inlineStr">
         <is>
           <t>You'll never run out of firewood again.
-[Weapon | Range: Short | Delay: D (2.3x) | Slots: 3]
+[Weapon | Range: Short | Delay: D (1.95x) | Slots: 3]
 Innate: Phys Hit +10% | Earth Res +20</t>
         </is>
       </c>
@@ -3100,7 +3100,7 @@
       <c r="F72" t="inlineStr">
         <is>
           <t>Wooden hammer that makes you want to climb icy mountains.
-[Weapon | Range: Short | Delay: D+ (2.15x) | Slots: 4]
+[Weapon | Range: Short | Delay: D+ (1.85x) | Slots: 4]
 Innate: Normal attacks: Freeze chance (20%) | DEX +5% | Water Res +20 | Water Res +10</t>
         </is>
       </c>
@@ -3137,7 +3137,7 @@
       <c r="F73" t="inlineStr">
         <is>
           <t>War god's axe with unimaginable destructive power.
-[Weapon | Range: Short | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Short | Delay: D (1.95x) | Slots: 4]
 Innate: Physical ATK vs. Magic Beings +20% | Phys Hit +10% | Crit Rate +5%</t>
         </is>
       </c>
@@ -3174,7 +3174,7 @@
       <c r="F74" t="inlineStr">
         <is>
           <t>Put in a possessed doll's hands, this is a tool of slaughter.
-[Weapon | Range: Short | Delay: E+ (2.45x) | Slots: 3]
+[Weapon | Range: Short | Delay: E+ (2.05x) | Slots: 3]
 Innate: Physical ATK vs. Beasts +50% | Earth Res +50 | HP Regen +4%/turn</t>
         </is>
       </c>
@@ -3211,7 +3211,7 @@
       <c r="F75" t="inlineStr">
         <is>
           <t>Bearded warriors can't get enough of these axes.
-[Weapon | Range: Short | Delay: E+ (2.45x) | Slots: 3]
+[Weapon | Range: Short | Delay: E+ (2.05x) | Slots: 3]
 Innate: Physical ATK vs. Sea Creatures +100% | Water Magic +15% | Water Res +20</t>
         </is>
       </c>
@@ -3248,7 +3248,7 @@
       <c r="F76" t="inlineStr">
         <is>
           <t>Sickle so heavily adorned with bones, it's hard to hold the grip.
-[Weapon | Range: Short | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Short | Delay: D (1.95x) | Slots: 4]
 Innate: Physical ATK vs. Humans +50% | Bash Res +20 | DEX -10%</t>
         </is>
       </c>
@@ -3285,7 +3285,7 @@
       <c r="F77" t="inlineStr">
         <is>
           <t>Axe that can crack the earth, exclusively used for battle.
-[Weapon | Range: Short | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Short | Delay: D (1.95x) | Slots: 4]
 Innate: Normal attacks: Petrify chance (15%) | Phys Hit +10% | Phys DEF +10%</t>
         </is>
       </c>
@@ -3322,7 +3322,7 @@
       <c r="F78" t="inlineStr">
         <is>
           <t>Axe filled with ghostly power, allowing it to destroy anything.
-[Weapon | Range: Short | Delay: E+ (2.45x) | Slots: 4]
+[Weapon | Range: Short | Delay: E+ (2.05x) | Slots: 4]
 Innate: Earth Magic +15% | Phys ATK +10% | HP Regen +4%/turn | Nullify poison</t>
         </is>
       </c>
@@ -3359,7 +3359,7 @@
       <c r="F79" t="inlineStr">
         <is>
           <t>Golden hammer granted by a plump god.
-[Weapon | Range: Short | Delay: D+ (2.15x) | Slots: 4]
+[Weapon | Range: Short | Delay: D+ (1.85x) | Slots: 4]
 Innate: Normal attacks: 20% HP Drain | Equipment Drop Rate +25% | Phys Dodge +10%</t>
         </is>
       </c>
@@ -3396,7 +3396,7 @@
       <c r="F80" t="inlineStr">
         <is>
           <t>Hammer designed to flatten the battlefield against higher beings.
-[Weapon | Range: Short | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Short | Delay: D (1.95x) | Slots: 4]
 Innate: Physical ATK vs. Demons +100% | RES +10% | Damage Taken -10%</t>
         </is>
       </c>
@@ -3433,7 +3433,7 @@
       <c r="F81" t="inlineStr">
         <is>
           <t>Super dangerous magic axe that gives wielders the urge to destroy.
-[Weapon | Range: Short | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Short | Delay: D (1.95x) | Slots: 4]
 Innate: Normal attacks: Stun chance (20%) | Phys ATK +10% | Action Speed +10%</t>
         </is>
       </c>
@@ -3470,7 +3470,7 @@
       <c r="F82" t="inlineStr">
         <is>
           <t>A weapon that can freely manipulate the deaths of others.
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 4]
 Innate: Normal attacks: Slow chance (15%) | Damage -&gt; TP (10%) | HP Regen +4%/turn</t>
         </is>
       </c>
@@ -3507,7 +3507,7 @@
       <c r="F83" t="inlineStr">
         <is>
           <t>Huge axe that bashes enemies to death with its immense weight.
-[Weapon | Range: Short | Delay: F (2.9x) | Slots: 0]
+[Weapon | Range: Short | Delay: F (2.35x) | Slots: 0]
 Innate: Standard equipment without innate passive enchantments.</t>
         </is>
       </c>
@@ -3544,7 +3544,7 @@
       <c r="F84" t="inlineStr">
         <is>
           <t>Huge axe with an exceedingly large blade and massive power.
-[Weapon | Range: Short | Delay: F+ (2.75x) | Slots: 3]
+[Weapon | Range: Short | Delay: F+ (2.25x) | Slots: 3]
 Innate: DEF +5% | DEX +10% | INT -10%</t>
         </is>
       </c>
@@ -3581,7 +3581,7 @@
       <c r="F85" t="inlineStr">
         <is>
           <t>High-tech axe which experts can ride in order to move around.
-[Weapon | Range: Short | Delay: F+ (2.75x) | Slots: 4]
+[Weapon | Range: Short | Delay: F+ (2.25x) | Slots: 4]
 Innate: Normal attacks: Stun chance (20%) | Phys Hit +10% | Crit Rate +10%</t>
         </is>
       </c>
@@ -3618,7 +3618,7 @@
       <c r="F86" t="inlineStr">
         <is>
           <t>Heavy equipment meant to get you ripped, not rip a hole in somebody.
-[Weapon | Range: Short | Delay: F (2.9x) | Slots: 4]
+[Weapon | Range: Short | Delay: F (2.35x) | Slots: 4]
 Innate: DEF +10% | Action Speed -10% | Action Speed -10%</t>
         </is>
       </c>
@@ -3655,7 +3655,7 @@
       <c r="F87" t="inlineStr">
         <is>
           <t>Crude axe wielded by an earthy frontiersman.
-[Weapon | Range: Short | Delay: F+ (2.75x) | Slots: 4]
+[Weapon | Range: Short | Delay: F+ (2.25x) | Slots: 4]
 Innate: Earth Magic +15% | RES +10% | Phys Hit +10% | Phys DEF +5%</t>
         </is>
       </c>
@@ -3692,7 +3692,7 @@
       <c r="F88" t="inlineStr">
         <is>
           <t>Dangerous weapon. Will make wielders thirst for murder.
-[Weapon | Range: Short | Delay: F (2.9x) | Slots: 3]
+[Weapon | Range: Short | Delay: F (2.35x) | Slots: 3]
 Innate: Normal attacks: 20% HP Drain | DEF +5% | Phys Damage Taken -10%</t>
         </is>
       </c>
@@ -3729,7 +3729,7 @@
       <c r="F89" t="inlineStr">
         <is>
           <t>High-tech armament consisting of a rocket engine on a stick.
-[Weapon | Range: Short | Delay: E (2.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: E (2.15x) | Slots: 4]
 Innate: AGI +5% | Phys Hit +10% | Earth Res +50</t>
         </is>
       </c>
@@ -3766,7 +3766,7 @@
       <c r="F90" t="inlineStr">
         <is>
           <t>Life-reaping scythe once owned by the Grim Reaper.
-[Weapon | Range: Short | Delay: F+ (2.75x) | Slots: 4]
+[Weapon | Range: Short | Delay: F+ (2.25x) | Slots: 4]
 Innate: Normal attacks: Instakill chance (15%) | DEX +10% | INT -10%</t>
         </is>
       </c>
@@ -3803,7 +3803,7 @@
       <c r="F91" t="inlineStr">
         <is>
           <t>Massive serpentine hatchet. The blade is bigger than Fried is.
-[Weapon | Range: Short | Delay: F (2.9x) | Slots: 4]
+[Weapon | Range: Short | Delay: F (2.35x) | Slots: 4]
 Innate: Normal attacks: 20% TP Drain | DEF +10% | Aggro/Enmity +25%</t>
         </is>
       </c>
@@ -3840,7 +3840,7 @@
       <c r="F92" t="inlineStr">
         <is>
           <t>A weapon with a crescent blade on each end. Hark to the hook!
-[Weapon | Range: Short | Delay: E (2.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: E (2.15x) | Slots: 4]
 Innate: Max TP +10% | Damage Taken -10% | HP Regen +4%/turn</t>
         </is>
       </c>
@@ -3877,7 +3877,7 @@
       <c r="F93" t="inlineStr">
         <is>
           <t>A berserker's favorite weapon. Kills weaklings who attempt to wield it.
-[Weapon | Range: Short | Delay: F+ (2.75x) | Slots: 4]
+[Weapon | Range: Short | Delay: F+ (2.25x) | Slots: 4]
 Innate: Physical ATK vs. Humans +50% | AGI +10% | INT -10% | TP Regen +4/turn</t>
         </is>
       </c>
@@ -3914,7 +3914,7 @@
       <c r="F94" t="inlineStr">
         <is>
           <t>Oversized scissors that can cut the strings of destiny.
-[Weapon | Range: Short | Delay: E (2.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: E (2.15x) | Slots: 4]
 Innate: Normal attacks: Instakill chance (15%) | DEF +10% | DEX +10%</t>
         </is>
       </c>
@@ -3951,7 +3951,7 @@
       <c r="F95" t="inlineStr">
         <is>
           <t>Hulking warhammer soaked with sweat and the blood of barbarians.
-[Weapon | Range: Short | Delay: F+ (2.75x) | Slots: 4]
+[Weapon | Range: Short | Delay: F+ (2.25x) | Slots: 4]
 Innate: Phys Hit +10% | Crit Rate +10% | Action Speed +10%</t>
         </is>
       </c>
@@ -3988,7 +3988,7 @@
       <c r="F96" t="inlineStr">
         <is>
           <t>Kijin's axe that's said to have shattered a planet.
-[Weapon | Range: Short | Delay: F (2.9x) | Slots: 4]
+[Weapon | Range: Short | Delay: F (2.35x) | Slots: 4]
 Innate: Physical ATK vs. Demons +50% | DEF +10% | Action Speed +10% | Nullify stun</t>
         </is>
       </c>
@@ -4025,7 +4025,7 @@
       <c r="F97" t="inlineStr">
         <is>
           <t>Legendary hammer used by titans who sustain the world.
-[Weapon | Range: Short | Delay: E (2.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: E (2.15x) | Slots: 4]
 Innate: Crit Rate +10% | Bash Res +30 | TP Regen +4/turn</t>
         </is>
       </c>
@@ -4062,7 +4062,7 @@
       <c r="F98" t="inlineStr">
         <is>
           <t>Fearsome sickle made by an earth goddess to castrate her husband.
-[Weapon | Range: Short | Delay: F+ (2.75x) | Slots: 4]
+[Weapon | Range: Short | Delay: F+ (2.25x) | Slots: 4]
 Innate: Normal attacks: 50% HP Drain | Max TP +10% | DEX +10% | Nullify slow</t>
         </is>
       </c>
@@ -4099,7 +4099,7 @@
       <c r="F99" t="inlineStr">
         <is>
           <t>One-handed weapon specialized in stabbing.
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 0]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 0]
 Innate: Standard equipment without innate passive enchantments.</t>
         </is>
       </c>
@@ -4136,7 +4136,7 @@
       <c r="F100" t="inlineStr">
         <is>
           <t>Spear-like weapon wielded by a delusional knight errant.
-[Weapon | Range: Short | Delay: D+ (2.15x) | Slots: 3]
+[Weapon | Range: Short | Delay: D+ (1.85x) | Slots: 3]
 Innate: Max HP +5% | Max TP -10%</t>
         </is>
       </c>
@@ -4173,7 +4173,7 @@
       <c r="F101" t="inlineStr">
         <is>
           <t>Huge and powerful cylinder made for battle.
-[Weapon | Range: Short | Delay: D+ (2.15x) | Slots: 3]
+[Weapon | Range: Short | Delay: D+ (1.85x) | Slots: 3]
 Innate: Normal attacks: 20% HP Drain | Phys Hit +10% | Crit Rate +10%</t>
         </is>
       </c>
@@ -4210,7 +4210,7 @@
       <c r="F102" t="inlineStr">
         <is>
           <t>Just the right size and weight for knighting around with.
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 3]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 3]
 Innate: DEX +10% | AGI +5% | Enemy Crit -10%</t>
         </is>
       </c>
@@ -4247,7 +4247,7 @@
       <c r="F103" t="inlineStr">
         <is>
           <t>Super-sized fork that giants use for their meals.
-[Weapon | Range: Short | Delay: D+ (2.15x) | Slots: 4]
+[Weapon | Range: Short | Delay: D+ (1.85x) | Slots: 4]
 Innate: Physical ATK vs. Beasts +20% | Action Speed +10% | Fire Res +20</t>
         </is>
       </c>
@@ -4284,7 +4284,7 @@
       <c r="F104" t="inlineStr">
         <is>
           <t>The princess's favorite umbrella.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 4]
 Innate: Water Magic +15% | INT +10% | Chant Speed +15% | Damage Taken -5%</t>
         </is>
       </c>
@@ -4321,7 +4321,7 @@
       <c r="F105" t="inlineStr">
         <is>
           <t>A lance forged of the holy metal called electrum.
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 3]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 3]
 Innate: Physical ATK vs. Demons +20% | Action Speed +10% | Lightning Res +50</t>
         </is>
       </c>
@@ -4358,7 +4358,7 @@
       <c r="F106" t="inlineStr">
         <is>
           <t>Weapon that releases heat from its tip thanks to magic.
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 4]
 Innate: Fire Magic +15% | Crit Rate +10% | Action Speed +5% | Water Res +20</t>
         </is>
       </c>
@@ -4395,7 +4395,7 @@
       <c r="F107" t="inlineStr">
         <is>
           <t>Short-ranged weapon with some extra oomph in the barrel.
-[Weapon | Range: Short | Delay: D+ (2.15x) | Slots: 4]
+[Weapon | Range: Short | Delay: D+ (1.85x) | Slots: 4]
 Innate: Phys Hit +10% | Phys Hit +10% | Action Speed +10% | Stab Res +20</t>
         </is>
       </c>
@@ -4432,7 +4432,7 @@
       <c r="F108" t="inlineStr">
         <is>
           <t>Spear made out of a sacred unicorn's horn. Extremely light.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 3]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 3]
 Innate: Action Speed +10% | All Elem Res +15 | TP Regen +4/turn</t>
         </is>
       </c>
@@ -4469,7 +4469,7 @@
       <c r="F109" t="inlineStr">
         <is>
           <t>The blood-red lance of a knight cursed with lifelong popularity.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 4]
 Innate: Normal attacks: Instakill chance (15%) | RES +10% | AGI +10%</t>
         </is>
       </c>
@@ -4506,7 +4506,7 @@
       <c r="F110" t="inlineStr">
         <is>
           <t>Lance that saps stamina from the ones it stabs.
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 4]
 Innate: Normal attacks: 50% HP Drain | Phys Hit +10% | Crit Rate +10% | Earth Res +20</t>
         </is>
       </c>
@@ -4543,7 +4543,7 @@
       <c r="F111" t="inlineStr">
         <is>
           <t>You stick your arm into it up to the elbow. The whole thing spins.
-[Weapon | Range: Short | Delay: D+ (2.15x) | Slots: 4]
+[Weapon | Range: Short | Delay: D+ (1.85x) | Slots: 4]
 Innate: Physical ATK vs. Magic Beings +50% | Action Speed +10% | Stab Res +50</t>
         </is>
       </c>
@@ -4580,7 +4580,7 @@
       <c r="F112" t="inlineStr">
         <is>
           <t>Spear filled with a seal fairy's love and misfortunes.
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 4]
 Innate: Water Magic +15% | Normal attacks: Freeze chance (20%) | Water Res +50</t>
         </is>
       </c>
@@ -4617,7 +4617,7 @@
       <c r="F113" t="inlineStr">
         <is>
           <t>Odin's godly spear that pierces all.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 4]
 Innate: Lightning Magic +15% | DEX +10% | Action Speed +10% | TP Regen +4/turn</t>
         </is>
       </c>
@@ -4654,7 +4654,7 @@
       <c r="F114" t="inlineStr">
         <is>
           <t>Three-pronged harpoon used by a sea-god in war and fishing alike.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 4]
 Innate: Physical ATK vs. Sea Creatures +100% | Normal attacks: Poison chance (20%)</t>
         </is>
       </c>
@@ -4691,7 +4691,7 @@
       <c r="F115" t="inlineStr">
         <is>
           <t>Large and highly powerful double-handed lance. Difficult to wield.
-[Weapon | Range: Mid | Delay: E+ (2.45x) | Slots: 0]
+[Weapon | Range: Mid | Delay: E+ (2.05x) | Slots: 0]
 Innate: Standard equipment without innate passive enchantments.</t>
         </is>
       </c>
@@ -4728,7 +4728,7 @@
       <c r="F116" t="inlineStr">
         <is>
           <t>The weapon doesn't matter if you've got heart! ...Hopefully!
-[Weapon | Range: Mid | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Mid | Delay: C+ (1.60x) | Slots: 4]
 Innate: Phys Hit +10% | Phys Hit +5% | Phys DEF +5% | Fire Res -20</t>
         </is>
       </c>
@@ -4765,7 +4765,7 @@
       <c r="F117" t="inlineStr">
         <is>
           <t>Ideally suited for capturing criminals. Safe enough to store anywhere.
-[Weapon | Range: Mid | Delay: C (2.0x) | Slots: 3]
+[Weapon | Range: Mid | Delay: C (1.75x) | Slots: 3]
 Innate: DEX +10% | Enemy Crit -10%</t>
         </is>
       </c>
@@ -4802,7 +4802,7 @@
       <c r="F118" t="inlineStr">
         <is>
           <t>Weapon that's similar to a spear that eastern fighters like to use.
-[Weapon | Range: Mid | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Mid | Delay: D (1.95x) | Slots: 4]
 Innate: Phys Hit +10% | Phys DEF +10% | Phys Dodge +10% | Action Speed +10%</t>
         </is>
       </c>
@@ -4839,7 +4839,7 @@
       <c r="F119" t="inlineStr">
         <is>
           <t>Big lance that does extra damage to dragons.
-[Weapon | Range: Mid | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Mid | Delay: D (1.95x) | Slots: 4]
 Innate: Physical ATK vs. Dragons +20% | Phys DEF +10% | Action Speed +5%</t>
         </is>
       </c>
@@ -4876,7 +4876,7 @@
       <c r="F120" t="inlineStr">
         <is>
           <t>Extremely large spear that no average person could wield.
-[Weapon | Range: Mid | Delay: E (2.6x) | Slots: 4]
+[Weapon | Range: Mid | Delay: E (2.15x) | Slots: 4]
 Innate: Normal attacks: 50% HP Drain | DEF +5% | Crit Rate +10%</t>
         </is>
       </c>
@@ -4913,7 +4913,7 @@
       <c r="F121" t="inlineStr">
         <is>
           <t>Massive cross-shaped spear wielded by a brusque demon.
-[Weapon | Range: Mid | Delay: D+ (2.15x) | Slots: 4]
+[Weapon | Range: Mid | Delay: D+ (1.85x) | Slots: 4]
 Innate: Normal attacks: 10% TP Drain | RES +10% | DEX +5% | AGI +5%</t>
         </is>
       </c>
@@ -4950,7 +4950,7 @@
       <c r="F122" t="inlineStr">
         <is>
           <t>Spear loved by the god of trade and combat. Can even cut dragons.
-[Weapon | Range: Mid | Delay: E+ (2.45x) | Slots: 4]
+[Weapon | Range: Mid | Delay: E+ (2.05x) | Slots: 4]
 Innate: Physical ATK vs. Dragons +50% | Normal attacks: Silence chance (20%)</t>
         </is>
       </c>
@@ -4987,7 +4987,7 @@
       <c r="F123" t="inlineStr">
         <is>
           <t>Weapon in the shape of a heavy lance, designed to destroy a holy book.
-[Weapon | Range: Mid | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Mid | Delay: D (1.95x) | Slots: 4]
 Innate: Normal attacks: Paralysis chance (20%) | DEF +10% | Magic DEF +10%</t>
         </is>
       </c>
@@ -5024,7 +5024,7 @@
       <c r="F124" t="inlineStr">
         <is>
           <t>Famous spear that would slice a firefly that lands on its tip in two.
-[Weapon | Range: Mid | Delay: D+ (2.15x) | Slots: 4]
+[Weapon | Range: Mid | Delay: D+ (1.85x) | Slots: 4]
 Innate: DEF +5% | DEX +10% | AGI +10% | Crit Rate +10%</t>
         </is>
       </c>
@@ -5061,7 +5061,7 @@
       <c r="F125" t="inlineStr">
         <is>
           <t>Strange pole that can freely change its size.
-[Weapon | Range: Mid | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Mid | Delay: D (1.95x) | Slots: 4]
 Innate: Physical ATK vs. Apparitions +50% | Action Speed +10% | Wind Res +50</t>
         </is>
       </c>
@@ -5098,7 +5098,7 @@
       <c r="F126" t="inlineStr">
         <is>
           <t>Bloodthirsty spear that yearns only to deliver its cursed poison.
-[Weapon | Range: Mid | Delay: D+ (2.15x) | Slots: 4]
+[Weapon | Range: Mid | Delay: D+ (1.85x) | Slots: 4]
 Innate: Normal attacks: Poison chance (20%) | Magic DEF +10% | Crit Rate +10%</t>
         </is>
       </c>
@@ -5135,7 +5135,7 @@
       <c r="F127" t="inlineStr">
         <is>
           <t>Spear made of sea animal bones. Destroys its victims from the inside.
-[Weapon | Range: Mid | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Mid | Delay: D (1.95x) | Slots: 4]
 Innate: Normal attacks: Instakill chance (15%) | Max TP +10% | DEF +10%</t>
         </is>
       </c>
@@ -5172,7 +5172,7 @@
       <c r="F128" t="inlineStr">
         <is>
           <t>Extensible spear used by a battle-loving maiden. Keep stowed.
-[Weapon | Range: Mid | Delay: D+ (2.15x) | Slots: 4]
+[Weapon | Range: Mid | Delay: D+ (1.85x) | Slots: 4]
 Innate: Physical ATK vs. Sea Creatures +100% | DEX +10% | Action Speed +10%</t>
         </is>
       </c>
@@ -5209,7 +5209,7 @@
       <c r="F129" t="inlineStr">
         <is>
           <t>Lance of a demigod maiden. Enspelled to make it easier to wield.
-[Weapon | Range: Mid | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Mid | Delay: D (1.95x) | Slots: 4]
 Innate: Physical ATK vs. Demons +50% | AGI +10% | Crit Rate +10% | HP Regen +4%/turn</t>
         </is>
       </c>
@@ -5246,7 +5246,7 @@
       <c r="F130" t="inlineStr">
         <is>
           <t>The destroyer god's unfair spear. Allows normal attacks to pierce.
-[Weapon | Range: Mid | Delay: E+ (2.45x) | Slots: 4]
+[Weapon | Range: Mid | Delay: E+ (2.05x) | Slots: 4]
 Innate: Physical ATK vs. Dragons +100% | RES +10% | AGI +10%</t>
         </is>
       </c>
@@ -5283,7 +5283,7 @@
       <c r="F131" t="inlineStr">
         <is>
           <t>Spear left behind by the god who created land.
-[Weapon | Range: Mid | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Mid | Delay: C+ (1.60x) | Slots: 4]
 Innate: Physical ATK vs. Apparitions +50% | Normal attacks: 10% TP Drain</t>
         </is>
       </c>
@@ -5320,7 +5320,7 @@
       <c r="F132" t="inlineStr">
         <is>
           <t>Striking rod with spikes on the tip.
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 0]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 0]
 Innate: Standard equipment without innate passive enchantments.</t>
         </is>
       </c>
@@ -5357,7 +5357,7 @@
       <c r="F133" t="inlineStr">
         <is>
           <t>Punishment rod for transgressors. Use sparingly!
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 2]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 2]
 Innate: Max TP +5% | Magic DEF +5%</t>
         </is>
       </c>
@@ -5394,7 +5394,7 @@
       <c r="F134" t="inlineStr">
         <is>
           <t>Long-handled cleaning implement made of expensive wood and silk.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 2]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 2]
 Innate: Interrupt Rate -25%</t>
         </is>
       </c>
@@ -5431,7 +5431,7 @@
       <c r="F135" t="inlineStr">
         <is>
           <t>Twirl it! Spin it! Rotate it! There are so many options.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 3]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 3]
 Innate: Normal attacks: 10% TP Drain | Magic Dodge +10% | Enemy Crit -10%</t>
         </is>
       </c>
@@ -5468,7 +5468,7 @@
       <c r="F136" t="inlineStr">
         <is>
           <t>Weapon loved by a lustful, excitable pig creature.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 3]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 3]
 Innate: Max HP +5% | Phys DEF +10% | Magic DEF +10%</t>
         </is>
       </c>
@@ -5505,7 +5505,7 @@
       <c r="F137" t="inlineStr">
         <is>
           <t>Regardless of the ingredients, nothing will burn or stick in this pan.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 3]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 3]
 Innate: Physical ATK vs. Fruit +50% | DEF +5% | Fire Res +20</t>
         </is>
       </c>
@@ -5542,7 +5542,7 @@
       <c r="F138" t="inlineStr">
         <is>
           <t>Ritual wand that can drive off evil or save the Seven Lucky Gods.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 3]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 3]
 Innate: Physical ATK vs. Apparitions +50% | Chant Speed +15% | TP Regen +4/turn</t>
         </is>
       </c>
@@ -5579,7 +5579,7 @@
       <c r="F139" t="inlineStr">
         <is>
           <t>Standard equipment for a maid robot.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 4]
 Innate: Max TP +10% | DEX -10% | All stats +3</t>
         </is>
       </c>
@@ -5616,7 +5616,7 @@
       <c r="F140" t="inlineStr">
         <is>
           <t>A ladle loved by Yassa the ship ghost.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 4]
 Innate: Water Magic +15% | Normal attacks: 10% TP Drain | Enemy Crit -10%</t>
         </is>
       </c>
@@ -5653,7 +5653,7 @@
       <c r="F141" t="inlineStr">
         <is>
           <t>Two sturdy rods anointed with holy water and joined by a silver chain.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 3]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 3]
 Innate: Physical ATK vs. Demons +20% | AGI +5%</t>
         </is>
       </c>
@@ -5690,7 +5690,7 @@
       <c r="F142" t="inlineStr">
         <is>
           <t>Poisoned morningstar that bludgeons with three spiky iron balls.
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 4]
 Innate: Normal attacks: Poison chance (20%) | RES +10% | Phys Hit +10%</t>
         </is>
       </c>
@@ -5727,7 +5727,7 @@
       <c r="F143" t="inlineStr">
         <is>
           <t>For a servant of God, that's a pretty brutal weapon...
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 4]
 Innate: Physical ATK vs. Demons +50% | Max TP +10% | Magic DEF +10%</t>
         </is>
       </c>
@@ -5764,7 +5764,7 @@
       <c r="F144" t="inlineStr">
         <is>
           <t>Bat made out of imaginary metal. Does that make the bat imaginary?
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 4]
 Innate: Normal attacks: Stun chance (20%) | INT +10% | RES +10% | AGI +5%</t>
         </is>
       </c>
@@ -5801,7 +5801,7 @@
       <c r="F145" t="inlineStr">
         <is>
           <t>Mace from the Three Sisters of Fate. Good against cats for some reason?
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 4]
 Innate: Physical ATK vs. Felines +100% | HP Regen +4%/turn | Nullify paralysis</t>
         </is>
       </c>
@@ -5838,7 +5838,7 @@
       <c r="F146" t="inlineStr">
         <is>
           <t>Lightning god's hammer. It crushes all that enters its path.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 4]
 Innate: Lightning Magic +15% | Max TP +10% | TP Regen +4/turn | Lightning Res +50</t>
         </is>
       </c>
@@ -5875,7 +5875,7 @@
       <c r="F147" t="inlineStr">
         <is>
           <t>Terrifying weapon that can control lightning.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 4]
 Innate: Lightning Magic +15% | Action Speed +10% | Chant Speed +15%</t>
         </is>
       </c>
@@ -5912,7 +5912,7 @@
       <c r="F148" t="inlineStr">
         <is>
           <t>Staff that increases the strength of magic attacks.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 0]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 0]
 Innate: Standard equipment without innate passive enchantments.</t>
         </is>
       </c>
@@ -5949,7 +5949,7 @@
       <c r="F149" t="inlineStr">
         <is>
           <t>Rod loved by the Dungeon Prez. Makes you a bit stupid(er).
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 3]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 3]
 Innate: Max HP +5% | DEX -10% | Aggro/Enmity -25%</t>
         </is>
       </c>
@@ -5986,7 +5986,7 @@
       <c r="F150" t="inlineStr">
         <is>
           <t>Staff with a talking bird on the tip. Very noisy.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 3]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 3]
 Innate: Magic Hit +10% | Magic Dodge +5% | Enemy Crit -10%</t>
         </is>
       </c>
@@ -6023,7 +6023,7 @@
       <c r="F151" t="inlineStr">
         <is>
           <t>Has a yellow heart on the end. See how it spins!
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 3]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 3]
 Innate: Normal attacks: 10% TP Drain | Max TP +5% | Magic Hit +10%</t>
         </is>
       </c>
@@ -6060,7 +6060,7 @@
       <c r="F152" t="inlineStr">
         <is>
           <t>Staff used to great effect by the mute magician Foley.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 4]
 Innate: Normal attacks: Silence chance (20%) | Max TP +10% | Magic DEF +10%</t>
         </is>
       </c>
@@ -6097,7 +6097,7 @@
       <c r="F153" t="inlineStr">
         <is>
           <t>Striking the enemy with this will emit electricity and stun them.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 3]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 3]
 Innate: Normal attacks: Stun chance (20%) | Phys ATK +10% | Magic ATK +10%</t>
         </is>
       </c>
@@ -6134,7 +6134,7 @@
       <c r="F154" t="inlineStr">
         <is>
           <t>Flexible wand with seven starry decorations.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 3]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 3]
 Innate: Damage -&gt; TP (10%) | TP Regen +4/turn | Earth Res +50</t>
         </is>
       </c>
@@ -6171,7 +6171,7 @@
       <c r="F155" t="inlineStr">
         <is>
           <t>Rod encrusted with a magical blue crystal.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 4]
 Innate: Max TP +10% | Magic Hit +10% | Magic Hit +10% | Chant Speed +15%</t>
         </is>
       </c>
@@ -6208,7 +6208,7 @@
       <c r="F156" t="inlineStr">
         <is>
           <t>Staff of fairy silver. Wrought by special magic and capped with a blade.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 4]
 Innate: Phys ATK +10% | Phys Hit +10% | Action Speed +10%</t>
         </is>
       </c>
@@ -6245,7 +6245,7 @@
       <c r="F157" t="inlineStr">
         <is>
           <t>Stafflike weapon of a kappa who joined a quest in search of sutras.
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 4]
 Innate: Max TP +10% | Magic DEF +10% | Chant Speed +15% | Magic Damage Taken -10%</t>
         </is>
       </c>
@@ -6282,7 +6282,7 @@
       <c r="F158" t="inlineStr">
         <is>
           <t>Staff owned by a demon who's some kind of a bigshot downstairs.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 4]
 Innate: Earth Magic +15% | Max TP +10% | Action Speed +10% | Interrupt Rate -50%</t>
         </is>
       </c>
@@ -6319,7 +6319,7 @@
       <c r="F159" t="inlineStr">
         <is>
           <t>Useful rod that can utilize the powers of both sun and moon.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 4]
 Innate: Max TP +10% | Interrupt Rate -90% | Fire Res +20 | Earth Res +20</t>
         </is>
       </c>
@@ -6356,7 +6356,7 @@
       <c r="F160" t="inlineStr">
         <is>
           <t>With love, pluck, and friendship, even a magic user can fight in front!
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 4]
 Innate: Phys ATK +10% | Magic ATK +10% | Damage -&gt; TP (10%)</t>
         </is>
       </c>
@@ -6393,7 +6393,7 @@
       <c r="F161" t="inlineStr">
         <is>
           <t>Charged with the power of the sun god. Comes with a free jade bead.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 4]
 Innate: Fire Magic +15% | Magic ATK +10% | Chant Speed +15% | Fire Res +50</t>
         </is>
       </c>
@@ -6430,7 +6430,7 @@
       <c r="F162" t="inlineStr">
         <is>
           <t>Ritual elephant goad. Very auspicious (unless you're an elephant).
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 4]
 Innate: Normal attacks: 20% TP Drain | Action Speed +10% | Chant Speed +15%</t>
         </is>
       </c>
@@ -6467,7 +6467,7 @@
       <c r="F163" t="inlineStr">
         <is>
           <t>Rod that was owned by the spirit Myrddin.
-[Weapon | Range: Short | Delay: A (1.2x) | Slots: 4]
+[Weapon | Range: Short | Delay: A (1.15x) | Slots: 4]
 Innate: Normal attacks: 20% TP Drain | Action Speed +10% | Chant Speed +15%</t>
         </is>
       </c>
@@ -6504,7 +6504,7 @@
       <c r="F164" t="inlineStr">
         <is>
           <t>Rod showered with the power to bestow fertility upon the land.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 4]
 Innate: Magic ATK +10% | Chant Speed +15% | Fully recover TP after battle</t>
         </is>
       </c>
@@ -6541,7 +6541,7 @@
       <c r="F165" t="inlineStr">
         <is>
           <t>Book stored with healing powers.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 0]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 0]
 Innate: Standard equipment without innate passive enchantments.</t>
         </is>
       </c>
@@ -6578,7 +6578,7 @@
       <c r="F166" t="inlineStr">
         <is>
           <t>Lurid, licentious, and vile.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 3]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 3]
 Innate: INT -10% | Interrupt Rate +25% | TP Regen +2/turn</t>
         </is>
       </c>
@@ -6615,7 +6615,7 @@
       <c r="F167" t="inlineStr">
         <is>
           <t>It was free. Don't complain.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 3]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 3]
 Innate: Pep is fixed at the minimum value | All Elem Res -30 | All Phys Res +50</t>
         </is>
       </c>
@@ -6652,7 +6652,7 @@
       <c r="F168" t="inlineStr">
         <is>
           <t>Encyclopedia that was gathering dust on the end of a bookshelf.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 2]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 2]
 Innate: Chant Speed +8% | TP Regen +4/turn</t>
         </is>
       </c>
@@ -6689,7 +6689,7 @@
       <c r="F169" t="inlineStr">
         <is>
           <t>Fundamental resource for any aspiring automata user.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 3]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 3]
 Innate: Max TP +10% | ATK +10% | Doll Potency +10%</t>
         </is>
       </c>
@@ -6726,7 +6726,7 @@
       <c r="F170" t="inlineStr">
         <is>
           <t>Diary that Athanasius had written in for years.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 4]
 Innate: Damage Taken -10% | Chant Speed +15% | HP Regen +2%/turn | TP Regen +2/turn</t>
         </is>
       </c>
@@ -6763,7 +6763,7 @@
       <c r="F171" t="inlineStr">
         <is>
           <t>Adventurous annals of ancient gods.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 4]
 Innate: Phys Damage Taken -10% | Earth Res +20 | Lightning Res +20</t>
         </is>
       </c>
@@ -6800,7 +6800,7 @@
       <c r="F172" t="inlineStr">
         <is>
           <t>Elohim essaim.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 4]
 Innate: Physical ATK vs. Beasts +20% | Magic Hit +10% | Magic Dodge +10%</t>
         </is>
       </c>
@@ -6837,7 +6837,7 @@
       <c r="F173" t="inlineStr">
         <is>
           <t>Tome written about summoning devils.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 4]
 Innate: Physical ATK vs. Demons +50% | Magic ATK +10% | Magic DEF +10%</t>
         </is>
       </c>
@@ -6874,7 +6874,7 @@
       <c r="F174" t="inlineStr">
         <is>
           <t>Open it and we're off on a fantastic adventure!
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 4]
 Innate: Interrupt Rate -50% | Phys Damage Taken -10% | Wind Res +20</t>
         </is>
       </c>
@@ -6911,7 +6911,7 @@
       <c r="F175" t="inlineStr">
         <is>
           <t>Book written about a promise with God.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 3]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 3]
 Innate: Normal attacks: Silence chance (20%) | TP Regen +2/turn | Nullify silence</t>
         </is>
       </c>
@@ -6948,7 +6948,7 @@
       <c r="F176" t="inlineStr">
         <is>
           <t>Pried from the chest of a freedom-loving giant metal lady.
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 4]
 Innate: Phys DEF +10% | Magic DEF +10% | Damage Taken -10% | HP Regen +4%/turn</t>
         </is>
       </c>
@@ -6985,7 +6985,7 @@
       <c r="F177" t="inlineStr">
         <is>
           <t>Black tome of wicked magicks penned by a vile sorcerer.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 4]
 Innate: Physical ATK vs. Humans +50% | Chant Speed +15% | TP Regen +4/turn</t>
         </is>
       </c>
@@ -7022,7 +7022,7 @@
       <c r="F178" t="inlineStr">
         <is>
           <t>Meticulous records of sinister dealings at the Casino Esperanza.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 4]
 Innate: Damage -&gt; TP (10%) | Nullify petrification | HP Regen +4%/turn</t>
         </is>
       </c>
@@ -7059,7 +7059,7 @@
       <c r="F179" t="inlineStr">
         <is>
           <t>Unspeakable text that enumerates scientific methods of murder.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 4]
 Innate: Max TP +10% | Magic ATK +10% | Chant Speed +15% | Doll Potency +10%</t>
         </is>
       </c>
@@ -7096,7 +7096,7 @@
       <c r="F180" t="inlineStr">
         <is>
           <t>Forbidden book that silences any struck by the corner of it.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 4]
 Innate: Physical ATK vs. Magic Beings +100% | AGI +10% | Nullify wind damage</t>
         </is>
       </c>
@@ -7133,7 +7133,7 @@
       <c r="F181" t="inlineStr">
         <is>
           <t>Small bow used for hunting.
-[Weapon | Range: Long | Delay: C+ (1.8x) | Slots: 0]
+[Weapon | Range: Long | Delay: C+ (1.60x) | Slots: 0]
 Innate: Standard equipment without innate passive enchantments.</t>
         </is>
       </c>
@@ -7170,7 +7170,7 @@
       <c r="F182" t="inlineStr">
         <is>
           <t>Sold as a souvenir at a place called the Eastern Shrine.
-[Weapon | Range: Long | Delay: C (2.0x) | Slots: 2]
+[Weapon | Range: Long | Delay: C (1.75x) | Slots: 2]
 Innate: Physical ATK vs. Apparitions +20% | Max TP +5%</t>
         </is>
       </c>
@@ -7207,7 +7207,7 @@
       <c r="F183" t="inlineStr">
         <is>
           <t>Bow wrapped in cherry tree bark and strung with whale tendons.
-[Weapon | Range: Long | Delay: C+ (1.8x) | Slots: 3]
+[Weapon | Range: Long | Delay: C+ (1.60x) | Slots: 3]
 Innate: Water Magic +15% | Physical ATK vs. Beasts +20% | Water Res +20</t>
         </is>
       </c>
@@ -7244,7 +7244,7 @@
       <c r="F184" t="inlineStr">
         <is>
           <t>Catalpa-wood bow. The string makes a pleasant sound when fired.
-[Weapon | Range: Long | Delay: B (1.6x) | Slots: 3]
+[Weapon | Range: Long | Delay: B (1.45x) | Slots: 3]
 Innate: Max TP +10% | DEX +5% | AGI +5%</t>
         </is>
       </c>
@@ -7281,7 +7281,7 @@
       <c r="F185" t="inlineStr">
         <is>
           <t>From this day forth, you're a hunter.
-[Weapon | Range: Long | Delay: B (1.6x) | Slots: 3]
+[Weapon | Range: Long | Delay: B (1.45x) | Slots: 3]
 Innate: DEX +10% | Phys Hit +10% | Crit Rate +10%</t>
         </is>
       </c>
@@ -7318,7 +7318,7 @@
       <c r="F186" t="inlineStr">
         <is>
           <t>Water bow born from the azure spring of intellect.
-[Weapon | Range: Long | Delay: C (2.0x) | Slots: 3]
+[Weapon | Range: Long | Delay: C (1.75x) | Slots: 3]
 Innate: Normal attacks: Freeze chance (20%) | Water Magic +15% | INT +10%</t>
         </is>
       </c>
@@ -7355,7 +7355,7 @@
       <c r="F187" t="inlineStr">
         <is>
           <t>True love will come if you aim for the heart.
-[Weapon | Range: Long | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Long | Delay: C+ (1.60x) | Slots: 4]
 Innate: Physical ATK vs. Humans +20% | Normal attacks: 20% HP Drain | Phys Hit +10%</t>
         </is>
       </c>
@@ -7392,7 +7392,7 @@
       <c r="F188" t="inlineStr">
         <is>
           <t>Bow beloved by a foolish, fey-touched bard.
-[Weapon | Range: Long | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Long | Delay: C+ (1.60x) | Slots: 4]
 Innate: Chant Speed +15% | Interrupt Rate -50% | TP Regen +4/turn | Song Potency +10%</t>
         </is>
       </c>
@@ -7429,7 +7429,7 @@
       <c r="F189" t="inlineStr">
         <is>
           <t>Bow used by a legendary apple hunter. It never misses.
-[Weapon | Range: Long | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Long | Delay: C+ (1.60x) | Slots: 4]
 Innate: Physical ATK vs. Fruit +50% | DEX +10% | Phys Hit +10% | Phys Hit +10%</t>
         </is>
       </c>
@@ -7466,7 +7466,7 @@
       <c r="F190" t="inlineStr">
         <is>
           <t>Bow that leaves a rainbow trail behind every shot.
-[Weapon | Range: Long | Delay: C+ (1.8x) | Slots: 3]
+[Weapon | Range: Long | Delay: C+ (1.60x) | Slots: 3]
 Innate: Normal attacks: 10% TP Drain | All Elem Res +15 | All Phys Res +15</t>
         </is>
       </c>
@@ -7503,7 +7503,7 @@
       <c r="F191" t="inlineStr">
         <is>
           <t>Usually enspelled to be small, it gets bigger when you ready it.
-[Weapon | Range: Long | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Long | Delay: B (1.45x) | Slots: 4]
 Innate: Max TP +10% | RES +10% | AGI +10% | Phys Dodge +10%</t>
         </is>
       </c>
@@ -7540,7 +7540,7 @@
       <c r="F192" t="inlineStr">
         <is>
           <t>The arrows this bow fires will even home in on moving targets.
-[Weapon | Range: Long | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Long | Delay: C+ (1.60x) | Slots: 4]
 Innate: DEX +10% | DEX +10% | Phys Hit +10%</t>
         </is>
       </c>
@@ -7577,7 +7577,7 @@
       <c r="F193" t="inlineStr">
         <is>
           <t>Horrible luck will befall whoever falls victim to this bow's strike.
-[Weapon | Range: Long | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Long | Delay: C (1.75x) | Slots: 4]
 Innate: Normal attacks: Stun chance (20%) | Max TP +10% | DEF +10%</t>
         </is>
       </c>
@@ -7614,7 +7614,7 @@
       <c r="F194" t="inlineStr">
         <is>
           <t>A strange energy shepherds the tips of its arrows through their targets.
-[Weapon | Range: Long | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Long | Delay: C (1.75x) | Slots: 4]
 Innate: Lightning Magic +15% | Magic ATK +10% | Chant Speed +15% | TP Regen +4/turn</t>
         </is>
       </c>
@@ -7651,7 +7651,7 @@
       <c r="F195" t="inlineStr">
         <is>
           <t>Splendorous bow of the chief of the cherubim. We're just borrowing it.
-[Weapon | Range: Long | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Long | Delay: C+ (1.60x) | Slots: 4]
 Innate: Physical ATK vs. Demons +50% | Action Speed +10% | Magic Damage Taken -10%</t>
         </is>
       </c>
@@ -7688,7 +7688,7 @@
       <c r="F196" t="inlineStr">
         <is>
           <t>Superweapon in the shape of a bow. Can wipe out a small country.
-[Weapon | Range: Long | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Long | Delay: B+ (1.30x) | Slots: 4]
 Innate: Fire Magic +15% | Physical ATK vs. Humans +100% | DEF +10% | Fire Res +30</t>
         </is>
       </c>
@@ -7725,7 +7725,7 @@
       <c r="F197" t="inlineStr">
         <is>
           <t>Large bow created for use in battle.
-[Weapon | Range: Long | Delay: E (2.6x) | Slots: 0]
+[Weapon | Range: Long | Delay: E (2.15x) | Slots: 0]
 Innate: Standard equipment without innate passive enchantments.</t>
         </is>
       </c>
@@ -7762,7 +7762,7 @@
       <c r="F198" t="inlineStr">
         <is>
           <t>Large bow that was enhanced to shoot even farther.
-[Weapon | Range: Long | Delay: F+ (2.75x) | Slots: 2]
+[Weapon | Range: Long | Delay: F+ (2.25x) | Slots: 2]
 Innate: DEX +5% | Crit Rate +10%</t>
         </is>
       </c>
@@ -7799,7 +7799,7 @@
       <c r="F199" t="inlineStr">
         <is>
           <t>Bow loved by forest fairies and showered with magic. And poison.
-[Weapon | Range: Long | Delay: E+ (2.45x) | Slots: 3]
+[Weapon | Range: Long | Delay: E+ (2.05x) | Slots: 3]
 Innate: Normal attacks: Poison chance (20%) | AGI +10% | Phys Hit +5%</t>
         </is>
       </c>
@@ -7836,7 +7836,7 @@
       <c r="F200" t="inlineStr">
         <is>
           <t>Wonderful for hunting. Less good for hitting targets.
-[Weapon | Range: Long | Delay: D (2.3x) | Slots: 3]
+[Weapon | Range: Long | Delay: D (1.95x) | Slots: 3]
 Innate: Phys Hit +10% | TP Regen +4/turn</t>
         </is>
       </c>
@@ -7873,7 +7873,7 @@
       <c r="F201" t="inlineStr">
         <is>
           <t>Large crossbow that can fire more than just arrows.
-[Weapon | Range: Long | Delay: E+ (2.45x) | Slots: 4]
+[Weapon | Range: Long | Delay: E+ (2.05x) | Slots: 4]
 Innate: DEF +5% | DEX +5% | Phys DEF +5% | Crit Rate +10%</t>
         </is>
       </c>
@@ -7910,7 +7910,7 @@
       <c r="F202" t="inlineStr">
         <is>
           <t>King's bow that appears in old heroic epics.
-[Weapon | Range: Long | Delay: E (2.6x) | Slots: 4]
+[Weapon | Range: Long | Delay: E (2.15x) | Slots: 4]
 Innate: Wind Magic +15% | DEF +5% | DEX +10% | Earth Res +20</t>
         </is>
       </c>
@@ -7947,7 +7947,7 @@
       <c r="F203" t="inlineStr">
         <is>
           <t>Empowered by a lightning spirit, its bolts hit home in a flash.
-[Weapon | Range: Long | Delay: E+ (2.45x) | Slots: 4]
+[Weapon | Range: Long | Delay: E+ (2.05x) | Slots: 4]
 Innate: Lightning Magic +15% | Max TP +10% | TP Regen +2/turn | Lightning Res +50</t>
         </is>
       </c>
@@ -7984,7 +7984,7 @@
       <c r="F204" t="inlineStr">
         <is>
           <t>Magical bow whose arrows reach into the heavenly blue sky.
-[Weapon | Range: Long | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Long | Delay: D (1.95x) | Slots: 4]
 Innate: Phys DEF +10% | Magic DEF +10% | HP Regen +4%/turn</t>
         </is>
       </c>
@@ -8021,7 +8021,7 @@
       <c r="F205" t="inlineStr">
         <is>
           <t>Large bow loved by a master archer. Crits like crazy.
-[Weapon | Range: Long | Delay: E (2.6x) | Slots: 4]
+[Weapon | Range: Long | Delay: E (2.15x) | Slots: 4]
 Innate: Max TP +10% | DEX +10% | Crit Rate +10% | Crit Rate +10%</t>
         </is>
       </c>
@@ -8058,7 +8058,7 @@
       <c r="F206" t="inlineStr">
         <is>
           <t>Godly bow received from the god of matchmaking.
-[Weapon | Range: Long | Delay: E+ (2.45x) | Slots: 4]
+[Weapon | Range: Long | Delay: E+ (2.05x) | Slots: 4]
 Innate: Normal attacks: 10% TP Drain | AGI +10% | Wind Res +50</t>
         </is>
       </c>
@@ -8095,7 +8095,7 @@
       <c r="F207" t="inlineStr">
         <is>
           <t>Disgusting bow of Nasu no Yoichi. Nasu-ty.
-[Weapon | Range: Long | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Long | Delay: D (1.95x) | Slots: 4]
 Innate: DEF +10% | All Elem Res +15 | All Phys Res +50 | TP Regen +4/turn</t>
         </is>
       </c>
@@ -8132,7 +8132,7 @@
       <c r="F208" t="inlineStr">
         <is>
           <t>Titan and draconic smithing turned a meteorite into a mighty bow.
-[Weapon | Range: Long | Delay: E+ (2.45x) | Slots: 4]
+[Weapon | Range: Long | Delay: E+ (2.05x) | Slots: 4]
 Innate: Wind Magic +15% | DEX +10% | Crit Rate +10% | Wind Res +50</t>
         </is>
       </c>
@@ -8169,7 +8169,7 @@
       <c r="F209" t="inlineStr">
         <is>
           <t>A weapon of the stony-gazed witch Medusa. Petrifyingly effective.
-[Weapon | Range: Long | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Long | Delay: C (1.75x) | Slots: 4]
 Innate: Normal attacks: Petrify chance (15%) | RES +10% | Magic Damage Taken -10%</t>
         </is>
       </c>
@@ -8206,7 +8206,7 @@
       <c r="F210" t="inlineStr">
         <is>
           <t>Holding this bow will make you want to hunt for boar.
-[Weapon | Range: Long | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Long | Delay: D (1.95x) | Slots: 4]
 Innate: DEF +10% | DEX +10% | AGI +10%</t>
         </is>
       </c>
@@ -8243,7 +8243,7 @@
       <c r="F211" t="inlineStr">
         <is>
           <t>Bow that'll skewer anything, no matter how hard.
-[Weapon | Range: Long | Delay: E (2.6x) | Slots: 4]
+[Weapon | Range: Long | Delay: E (2.15x) | Slots: 4]
 Innate: Physical ATK vs. Beasts +50% | Normal attacks: Silence chance (20%)</t>
         </is>
       </c>
@@ -8280,7 +8280,7 @@
       <c r="F212" t="inlineStr">
         <is>
           <t>Godly bow with shocking power that reaches the heavens.
-[Weapon | Range: Long | Delay: E+ (2.45x) | Slots: 4]
+[Weapon | Range: Long | Delay: E+ (2.05x) | Slots: 4]
 Innate: Physical ATK vs. Demons +100% | TP Regen +4/turn | DEX +10% | AGI +10%</t>
         </is>
       </c>
@@ -8317,7 +8317,7 @@
       <c r="F213" t="inlineStr">
         <is>
           <t>Short-chambered revolver. It's been looked after with love.
-[Weapon | Range: Long | Delay: B (1.6x) | Slots: 2]
+[Weapon | Range: Long | Delay: B (1.45x) | Slots: 2]
 Innate: AGI +10% | Phys Hit +10%</t>
         </is>
       </c>
@@ -8354,7 +8354,7 @@
       <c r="F214" t="inlineStr">
         <is>
           <t>Handily hides in a pendant when not in use. Fires penetrating bullets.
-[Weapon | Range: Long | Delay: F+ (2.75x) | Slots: 4]
+[Weapon | Range: Long | Delay: F+ (2.25x) | Slots: 4]
 Innate: Phys Hit +10% | Crit Rate +10% | HP Regen +4%/turn | Action Speed -10%</t>
         </is>
       </c>
@@ -8391,7 +8391,7 @@
       <c r="F215" t="inlineStr">
         <is>
           <t>Elegant musket that fires magic bullets.
-[Weapon | Range: Mid | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Mid | Delay: D (1.95x) | Slots: 4]
 Innate: Physical ATK vs. Demons +20% | DEX +10% | Magic ATK +10% | TP Regen +4/turn</t>
         </is>
       </c>
@@ -8428,7 +8428,7 @@
       <c r="F216" t="inlineStr">
         <is>
           <t>Fires lasers of hyperconcentrated light. How does it work...?
-[Weapon | Range: Long | Delay: F+ (2.75x) | Slots: 4]
+[Weapon | Range: Long | Delay: F+ (2.25x) | Slots: 4]
 Innate: Physical ATK vs. Magic Beings +20% | DEF +10% | Phys Hit +10%</t>
         </is>
       </c>
@@ -8465,7 +8465,7 @@
       <c r="F217" t="inlineStr">
         <is>
           <t>Once you get the hang of it, you can shoot it with your eyes closed.
-[Weapon | Range: Mid | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Mid | Delay: B+ (1.30x) | Slots: 4]
 Innate: AGI +10% | Crit Rate +10% | Damage -&gt; TP (10%)</t>
         </is>
       </c>
@@ -8502,7 +8502,7 @@
       <c r="F218" t="inlineStr">
         <is>
           <t>Forbidden weapon that harnesses micro black holes and hypergravity.
-[Weapon | Range: Long | Delay: F (2.9x) | Slots: 4]
+[Weapon | Range: Long | Delay: F (2.35x) | Slots: 4]
 Innate: DEF +10% | Nullify stun | AGI -10%</t>
         </is>
       </c>
@@ -8539,7 +8539,7 @@
       <c r="F219" t="inlineStr">
         <is>
           <t>Gun made of orichalcum and built to kill god.
-[Weapon | Range: Long | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Long | Delay: D (1.95x) | Slots: 4]
 Innate: Physical ATK vs. Magic Beings +100% | Normal attacks: Stun chance (20%)</t>
         </is>
       </c>
@@ -8576,7 +8576,7 @@
       <c r="F220" t="inlineStr">
         <is>
           <t>Small, one-handed curved katana that came from an eastern country.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 0]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 0]
 Innate: Standard equipment without innate passive enchantments.</t>
         </is>
       </c>
@@ -8613,7 +8613,7 @@
       <c r="F221" t="inlineStr">
         <is>
           <t>Long katana with no guard favored by four-fingered samurai.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 3]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 3]
 Innate: Physical ATK vs. Humans +20% | Crit Rate +10% | Aggro/Enmity +25%</t>
         </is>
       </c>
@@ -8650,7 +8650,7 @@
       <c r="F222" t="inlineStr">
         <is>
           <t>Gunmetal gray sword that gives an advantage in nocturnal duels.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 4]
 Innate: Phys Hit +10% | Phys Dodge +10% | Magic Dodge +10% | Enemy Crit -10%</t>
         </is>
       </c>
@@ -8687,7 +8687,7 @@
       <c r="F223" t="inlineStr">
         <is>
           <t>Katana that's said to weaken apparitional powers.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 3]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 3]
 Innate: Physical ATK vs. Apparitions +20% | HP Regen +4%/turn | TP Regen +2/turn</t>
         </is>
       </c>
@@ -8724,7 +8724,7 @@
       <c r="F224" t="inlineStr">
         <is>
           <t>Handy katana that sometimes knocks out those it cuts.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 3]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 3]
 Innate: Normal attacks: Stun chance (20%) | Phys Hit +10% | Phys Dodge +10%</t>
         </is>
       </c>
@@ -8761,7 +8761,7 @@
       <c r="F225" t="inlineStr">
         <is>
           <t>Tantou used by a country's naval units.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 4]
 Innate: Water Magic +15% | Normal attacks: Poison chance (20%) | DEX +5% | AGI +5%</t>
         </is>
       </c>
@@ -8798,7 +8798,7 @@
       <c r="F226" t="inlineStr">
         <is>
           <t>Good, sharp wakizashi with a regrettable tendency to doom its user.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 4]
 Innate: AGI +5% | Damage -&gt; TP (10%) | Max HP -10% | Aggro/Enmity +25%</t>
         </is>
       </c>
@@ -8835,7 +8835,7 @@
       <c r="F227" t="inlineStr">
         <is>
           <t>It yearns to cut whoever comes into its path.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 4]
 Innate: Normal attacks: Slow chance (15%) | DEX +10% | Phys Dodge +10% | Fire Res -20</t>
         </is>
       </c>
@@ -8872,7 +8872,7 @@
       <c r="F228" t="inlineStr">
         <is>
           <t>Rare tantou with a curved blade. Flexible and tough to break.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 3]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 3]
 Innate: AGI +5% | Crit Rate +10%</t>
         </is>
       </c>
@@ -8909,7 +8909,7 @@
       <c r="F229" t="inlineStr">
         <is>
           <t>Ninja blade brought to the big city by a ninja from the Koga boondocks.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 4]
 Innate: Phys ATK +10% | Phys Dodge +10% | Nullify gas traps | Lightning Res -20</t>
         </is>
       </c>
@@ -8946,7 +8946,7 @@
       <c r="F230" t="inlineStr">
         <is>
           <t>Ninja katana once owned by a chivalrous young thief.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 4]
 Innate: Fire Magic +15% | Normal attacks: Stun chance (20%) | Crit Rate +10%</t>
         </is>
       </c>
@@ -8983,7 +8983,7 @@
       <c r="F231" t="inlineStr">
         <is>
           <t>Katana that can be wielded with such grace, it can slice lightning.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 4]
 Innate: Lightning Magic +15% | Action Speed +10% | Chant Speed +15% | Slash Res +20</t>
         </is>
       </c>
@@ -9020,7 +9020,7 @@
       <c r="F232" t="inlineStr">
         <is>
           <t>Splendidly sharp tantou created by master craftsman Yoshimitsu.
-[Weapon | Range: Short | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: B (1.45x) | Slots: 4]
 Innate: Normal attacks: Stun chance (20%) | RES +10% | DEX +10% | AGI +10%</t>
         </is>
       </c>
@@ -9057,7 +9057,7 @@
       <c r="F233" t="inlineStr">
         <is>
           <t>Katana that can cut ghosts and sweep away ghostly atmospheres.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 4]
 Innate: Physical ATK vs. Apparitions +50% | DEF +5% | Phys Dodge +10%</t>
         </is>
       </c>
@@ -9094,7 +9094,7 @@
       <c r="F234" t="inlineStr">
         <is>
           <t>Cursed blade that severs anything it cuts. Clean with caution.
-[Weapon | Range: Short | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Short | Delay: B+ (1.30x) | Slots: 4]
 Innate: Normal attacks: High Instakill chance (50%) | DEX +10% | Crit Rate +10%</t>
         </is>
       </c>
@@ -9131,7 +9131,7 @@
       <c r="F235" t="inlineStr">
         <is>
           <t>Ninja katana loved by Jiraiya, the legendary ninja.
-[Weapon | Range: Short | Delay: A (1.2x) | Slots: 4]
+[Weapon | Range: Short | Delay: A (1.15x) | Slots: 4]
 Innate: Physical ATK vs. Apparitions +100% | Phys Dodge +10% | Action Speed +10%</t>
         </is>
       </c>
@@ -9168,7 +9168,7 @@
       <c r="F236" t="inlineStr">
         <is>
           <t>Large, two-handed curved katana that eastern warriors like to use.
-[Weapon | Range: Short | Delay: E (2.6x) | Slots: 0]
+[Weapon | Range: Short | Delay: E (2.15x) | Slots: 0]
 Innate: Standard equipment without innate passive enchantments.</t>
         </is>
       </c>
@@ -9205,7 +9205,7 @@
       <c r="F237" t="inlineStr">
         <is>
           <t>Ritual sword created to communicate with God. Can also sorta cut.
-[Weapon | Range: Short | Delay: E+ (2.45x) | Slots: 3]
+[Weapon | Range: Short | Delay: E+ (2.05x) | Slots: 3]
 Innate: RES +10% | Phys Hit +5%</t>
         </is>
       </c>
@@ -9242,7 +9242,7 @@
       <c r="F238" t="inlineStr">
         <is>
           <t>Katana once wielded by a proud Evenkuruga.
-[Weapon | Range: Short | Delay: E (2.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: E (2.15x) | Slots: 4]
 Innate: Water Magic +15% | DEF +10% | Crit Rate +10% | Aggro/Enmity +25%</t>
         </is>
       </c>
@@ -9279,7 +9279,7 @@
       <c r="F239" t="inlineStr">
         <is>
           <t>Sword of dominance used by an army's special forces.
-[Weapon | Range: Short | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Short | Delay: D (1.95x) | Slots: 4]
 Innate: Fire Magic +15% | Action Speed +10% | Action Speed +5% | TP Regen +4/turn</t>
         </is>
       </c>
@@ -9316,7 +9316,7 @@
       <c r="F240" t="inlineStr">
         <is>
           <t>Tachi too long for even most samurai to wield.
-[Weapon | Range: Short | Delay: F+ (2.75x) | Slots: 4]
+[Weapon | Range: Short | Delay: F+ (2.25x) | Slots: 4]
 Innate: DEF +10% | Phys DEF +10% | Aggro/Enmity +25% | Action Speed -10%</t>
         </is>
       </c>
@@ -9353,7 +9353,7 @@
       <c r="F241" t="inlineStr">
         <is>
           <t>A light katana that can provide multiple attacks.
-[Weapon | Range: Short | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Short | Delay: D (1.95x) | Slots: 4]
 Innate: DEX +10% | AGI +5% | Phys Dodge +10%</t>
         </is>
       </c>
@@ -9390,7 +9390,7 @@
       <c r="F242" t="inlineStr">
         <is>
           <t>Bewitched sword in which a tsuruhime spirit dwells. Quite sharp.
-[Weapon | Range: Short | Delay: E+ (2.45x) | Slots: 4]
+[Weapon | Range: Short | Delay: E+ (2.05x) | Slots: 4]
 Innate: Physical ATK vs. Apparitions +50% | Phys DEF +10% | Magic DEF +10%</t>
         </is>
       </c>
@@ -9427,7 +9427,7 @@
       <c r="F243" t="inlineStr">
         <is>
           <t>Tachi with beautiful crescent-moon forging patterns.
-[Weapon | Range: Short | Delay: E+ (2.45x) | Slots: 4]
+[Weapon | Range: Short | Delay: E+ (2.05x) | Slots: 4]
 Innate: DEF +10% | Phys Dodge +10% | Slash Res +20</t>
         </is>
       </c>
@@ -9464,7 +9464,7 @@
       <c r="F244" t="inlineStr">
         <is>
           <t>Tachi said to be capable of cutting stone and splitting helmets.
-[Weapon | Range: Short | Delay: E (2.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: E (2.15x) | Slots: 4]
 Innate: Physical ATK vs. Humans +50% | Action Speed +10% | HP Regen +4%/turn</t>
         </is>
       </c>
@@ -9501,7 +9501,7 @@
       <c r="F245" t="inlineStr">
         <is>
           <t>A tachi so sharp, the victim won't even notice the cut.
-[Weapon | Range: Short | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Short | Delay: D (1.95x) | Slots: 4]
 Innate: AGI +10% | Phys ATK +10% | Phys Hit +10%</t>
         </is>
       </c>
@@ -9538,7 +9538,7 @@
       <c r="F246" t="inlineStr">
         <is>
           <t>Katana of a famous vice-commander who fought like a demon to the last.
-[Weapon | Range: Short | Delay: E+ (2.45x) | Slots: 4]
+[Weapon | Range: Short | Delay: E+ (2.05x) | Slots: 4]
 Innate: Normal attacks: Instakill chance (15%) | DEX +10% | Phys DEF +10%</t>
         </is>
       </c>
@@ -9575,7 +9575,7 @@
       <c r="F247" t="inlineStr">
         <is>
           <t>Slender light tachi with lacquerwork lions on its scabbard.
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 4]
 Innate: RES +10% | Action Speed +10% | Magic Damage Taken -10% | TP Regen +4/turn</t>
         </is>
       </c>
@@ -9612,7 +9612,7 @@
       <c r="F248" t="inlineStr">
         <is>
           <t>Huge tachi for slaying apparitions. Flies at spectral presences on its own.
-[Weapon | Range: Short | Delay: F (2.9x) | Slots: 4]
+[Weapon | Range: Short | Delay: F (2.35x) | Slots: 4]
 Innate: Physical ATK vs. Apparitions +50% | Max TP +10% | RES +10%</t>
         </is>
       </c>
@@ -9649,7 +9649,7 @@
       <c r="F249" t="inlineStr">
         <is>
           <t>Bewitched katana with a shady history involving the shogunate.
-[Weapon | Range: Short | Delay: E (2.6x) | Slots: 4]
+[Weapon | Range: Short | Delay: E (2.15x) | Slots: 4]
 Innate: Normal attacks: 10% TP Drain | Crit Rate +10% | Action Speed +10%</t>
         </is>
       </c>
@@ -9686,7 +9686,7 @@
       <c r="F250" t="inlineStr">
         <is>
           <t>Devil sword that yells in the night about its thirst for blood.
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 4]
 Innate: Normal attacks: Silence chance (20%) | Physical ATK vs. Humans +100%</t>
         </is>
       </c>
@@ -9723,7 +9723,7 @@
       <c r="F251" t="inlineStr">
         <is>
           <t>Original tachi complete with ultimate sharpness and beauty.
-[Weapon | Range: Short | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Short | Delay: D (1.95x) | Slots: 4]
 Innate: Normal attacks: Petrify chance (15%) | Max TP +10% | AGI +10%</t>
         </is>
       </c>
@@ -9760,7 +9760,7 @@
       <c r="F252" t="inlineStr">
         <is>
           <t>Projectiles with needles on the tip.
-[Weapon | Range: Long | Delay: B (1.6x) | Slots: 0]
+[Weapon | Range: Long | Delay: B (1.45x) | Slots: 0]
 Innate: Standard equipment without innate passive enchantments.</t>
         </is>
       </c>
@@ -9797,7 +9797,7 @@
       <c r="F253" t="inlineStr">
         <is>
           <t>Knife with feathers tied to it to help it fly.
-[Weapon | Range: Long | Delay: B (1.6x) | Slots: 3]
+[Weapon | Range: Long | Delay: B (1.45x) | Slots: 3]
 Innate: Crit Rate +10% | Wind Res +20 | Earth Res -20</t>
         </is>
       </c>
@@ -9834,7 +9834,7 @@
       <c r="F254" t="inlineStr">
         <is>
           <t>A sake bottle with flammable liquid inside.
-[Weapon | Range: Long | Delay: C (2.0x) | Slots: 2]
+[Weapon | Range: Long | Delay: C (1.75x) | Slots: 2]
 Innate: Fire Magic +15% | Water Res -20</t>
         </is>
       </c>
@@ -9871,7 +9871,7 @@
       <c r="F255" t="inlineStr">
         <is>
           <t>Throwing needle doused with copious anesthetics.
-[Weapon | Range: Long | Delay: B (1.6x) | Slots: 2]
+[Weapon | Range: Long | Delay: B (1.45x) | Slots: 2]
 Innate: Normal attacks: Sleep chance (20%) | Action Speed +10%</t>
         </is>
       </c>
@@ -9908,7 +9908,7 @@
       <c r="F256" t="inlineStr">
         <is>
           <t>Regulation kunoichi kit. Big enough to use hand-to-hand too.
-[Weapon | Range: Long | Delay: C+ (1.8x) | Slots: 3]
+[Weapon | Range: Long | Delay: C+ (1.60x) | Slots: 3]
 Innate: Normal attacks: Instakill chance (15%) | AGI +10% | Phys Dodge +5%</t>
         </is>
       </c>
@@ -9945,7 +9945,7 @@
       <c r="F257" t="inlineStr">
         <is>
           <t>Magical arrow with an automatic homing system.
-[Weapon | Range: Long | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Long | Delay: B (1.45x) | Slots: 4]
 Innate: DEX +10% | Phys Hit +10% | Phys Hit +10% | Action Speed +5%</t>
         </is>
       </c>
@@ -9982,7 +9982,7 @@
       <c r="F258" t="inlineStr">
         <is>
           <t>Pitch black kunai. Dangerous when thrown in the darkness.
-[Weapon | Range: Long | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Long | Delay: B+ (1.30x) | Slots: 4]
 Innate: Normal attacks: Instakill chance (15%) | Crit Rate +10% | Enemy Crit -10%</t>
         </is>
       </c>
@@ -10019,7 +10019,7 @@
       <c r="F259" t="inlineStr">
         <is>
           <t>Projectile weapon shaped like a rose. Won't come off once it's stuck.
-[Weapon | Range: Long | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Long | Delay: B (1.45x) | Slots: 4]
 Innate: Normal attacks: Poison chance (20%) | Crit Rate +10% | Action Speed +10%</t>
         </is>
       </c>
@@ -10056,7 +10056,7 @@
       <c r="F260" t="inlineStr">
         <is>
           <t>Playing cards made out of extremely precious metal.
-[Weapon | Range: Long | Delay: B+ (1.4x) | Slots: 3]
+[Weapon | Range: Long | Delay: B+ (1.30x) | Slots: 3]
 Innate: HP Regen +4%/turn | TP Regen +4/turn | Pep will not drop below 100</t>
         </is>
       </c>
@@ -10093,7 +10093,7 @@
       <c r="F261" t="inlineStr">
         <is>
           <t>Hard, sharp card loaded with kinetic energy.
-[Weapon | Range: Long | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Long | Delay: B (1.45x) | Slots: 4]
 Innate: Wind Magic +15% | All stats +3 | Action Speed +10% | Wind Res +20</t>
         </is>
       </c>
@@ -10130,7 +10130,7 @@
       <c r="F262" t="inlineStr">
         <is>
           <t>Chakram that'll continue to fly round until the enemy is defeated.
-[Weapon | Range: Long | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Long | Delay: C+ (1.60x) | Slots: 4]
 Innate: Physical ATK vs. Dragons +50% | AGI +10% | Crit Rate +10% | Action Speed +10%</t>
         </is>
       </c>
@@ -10167,7 +10167,7 @@
       <c r="F263" t="inlineStr">
         <is>
           <t>Head-mounted boomerang. It's important to yell when you throw it.
-[Weapon | Range: Long | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Long | Delay: C+ (1.60x) | Slots: 4]
 Innate: Physical ATK vs. Beasts +50% | Phys Hit +10% | All Elem Res +15</t>
         </is>
       </c>
@@ -10204,7 +10204,7 @@
       <c r="F264" t="inlineStr">
         <is>
           <t>Shuriken that the Fuma clan created with malice.
-[Weapon | Range: Long | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Long | Delay: B (1.45x) | Slots: 4]
 Innate: Physical ATK vs. Apparitions +50% | Normal attacks: Paralysis chance (20%)</t>
         </is>
       </c>
@@ -10241,7 +10241,7 @@
       <c r="F265" t="inlineStr">
         <is>
           <t>Disc that harnesses magnetic force to fly both far and fast.
-[Weapon | Range: Long | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Long | Delay: C (1.75x) | Slots: 4]
 Innate: Max HP +5% | Max TP +5% | Phys Dodge +10% | Crit Rate +10%</t>
         </is>
       </c>
@@ -10278,7 +10278,7 @@
       <c r="F266" t="inlineStr">
         <is>
           <t>Kunai that the legendary kunoichi Tsunade loved to use.
-[Weapon | Range: Long | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Long | Delay: B (1.45x) | Slots: 4]
 Innate: Physical ATK vs. Apparitions +50% | Action Speed +10% | Chant Speed +15%</t>
         </is>
       </c>
@@ -10315,7 +10315,7 @@
       <c r="F267" t="inlineStr">
         <is>
           <t>Chakram that hits home and flies back on its own.
-[Weapon | Range: Long | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Long | Delay: C+ (1.60x) | Slots: 4]
 Innate: Normal attacks: Slow chance (15%) | DEF +10% | Crit Rate +10% | Stab Res +50</t>
         </is>
       </c>
@@ -10352,7 +10352,7 @@
       <c r="F268" t="inlineStr">
         <is>
           <t>Blade of light that won't stop until it pierces an enemy.
-[Weapon | Range: Long | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Long | Delay: B+ (1.30x) | Slots: 4]
 Innate: Physical ATK vs. Demons +50% | Max TP +10% | Phys Hit +10%</t>
         </is>
       </c>
@@ -10389,7 +10389,7 @@
       <c r="F269" t="inlineStr">
         <is>
           <t>Whip that is best suited for mid-range attacks to the enemies.
-[Weapon | Range: Mid | Delay: D (2.3x) | Slots: 0]
+[Weapon | Range: Mid | Delay: D (1.95x) | Slots: 0]
 Innate: Standard equipment without innate passive enchantments.</t>
         </is>
       </c>
@@ -10426,7 +10426,7 @@
       <c r="F270" t="inlineStr">
         <is>
           <t>Whip used for punishment. Teachers and such love to use them.
-[Weapon | Range: Mid | Delay: D (2.3x) | Slots: 2]
+[Weapon | Range: Mid | Delay: D (1.95x) | Slots: 2]
 Innate: Phys Hit +10% | Crit Rate +10%</t>
         </is>
       </c>
@@ -10463,7 +10463,7 @@
       <c r="F271" t="inlineStr">
         <is>
           <t>Whip for hitting horses. Strike it too much and it'll throw you off.
-[Weapon | Range: Mid | Delay: D+ (2.15x) | Slots: 3]
+[Weapon | Range: Mid | Delay: D+ (1.85x) | Slots: 3]
 Innate: Physical ATK vs. Beasts +20% | Phys Dodge +10% | Aggro/Enmity +25%</t>
         </is>
       </c>
@@ -10500,7 +10500,7 @@
       <c r="F272" t="inlineStr">
         <is>
           <t>Whip crafted by sadists for the ultimate play.
-[Weapon | Range: Mid | Delay: D+ (2.15x) | Slots: 3]
+[Weapon | Range: Mid | Delay: D+ (1.85x) | Slots: 3]
 Innate: Normal attacks: 20% HP Drain | DEF +5% | AGI +10%</t>
         </is>
       </c>
@@ -10537,7 +10537,7 @@
       <c r="F273" t="inlineStr">
         <is>
           <t>Whip made for torture. Skin will split, and blood will trickle.
-[Weapon | Range: Mid | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Mid | Delay: D (1.95x) | Slots: 4]
 Innate: Max TP +10% | Phys ATK +10% | Enemy Crit -10% | Aggro/Enmity +25%</t>
         </is>
       </c>
@@ -10574,7 +10574,7 @@
       <c r="F274" t="inlineStr">
         <is>
           <t>All-purpose whip that belongs in a museum.
-[Weapon | Range: Mid | Delay: D+ (2.15x) | Slots: 4]
+[Weapon | Range: Mid | Delay: D+ (1.85x) | Slots: 4]
 Innate: Earth Magic +15% | DEX +10% | Aggro/Enmity -25% | Earth Res +20</t>
         </is>
       </c>
@@ -10611,7 +10611,7 @@
       <c r="F275" t="inlineStr">
         <is>
           <t>Red-white rope once hung around a sacred tree.
-[Weapon | Range: Mid | Delay: D+ (2.15x) | Slots: 4]
+[Weapon | Range: Mid | Delay: D+ (1.85x) | Slots: 4]
 Innate: Song Potency +10% | Dance Potency +10% | Doll Potency +10%</t>
         </is>
       </c>
@@ -10648,7 +10648,7 @@
       <c r="F276" t="inlineStr">
         <is>
           <t>Pain is love! Pain is peace! Pain is pleasure!
-[Weapon | Range: Mid | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Mid | Delay: D (1.95x) | Slots: 4]
 Innate: Normal attacks: 50% HP Drain | DEF +10% | Wind Res +20 | Earth Res +20</t>
         </is>
       </c>
@@ -10685,7 +10685,7 @@
       <c r="F277" t="inlineStr">
         <is>
           <t>Whip that used to be a demon's tail. Smooth as silk.
-[Weapon | Range: Mid | Delay: E+ (2.45x) | Slots: 4]
+[Weapon | Range: Mid | Delay: E+ (2.05x) | Slots: 4]
 Innate: Normal attacks: 10% TP Drain | Damage -&gt; TP (10%) | TP Regen +4/turn</t>
         </is>
       </c>
@@ -10722,7 +10722,7 @@
       <c r="F278" t="inlineStr">
         <is>
           <t>Rubbery lash. Watch out for the suckers.
-[Weapon | Range: Mid | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Mid | Delay: C (1.75x) | Slots: 4]
 Innate: Normal attacks: Paralysis chance (20%) | Max TP +10% | AGI +10%</t>
         </is>
       </c>
@@ -10759,7 +10759,7 @@
       <c r="F279" t="inlineStr">
         <is>
           <t>Whip owned by the queen of the night. Kneel down and lick my shoes!
-[Weapon | Range: Mid | Delay: D (2.3x) | Slots: 3]
+[Weapon | Range: Mid | Delay: D (1.95x) | Slots: 3]
 Innate: Aggro/Enmity +25% | Pep is fixed at the max value</t>
         </is>
       </c>
@@ -10796,7 +10796,7 @@
       <c r="F280" t="inlineStr">
         <is>
           <t>Magical whip that creates crimson flames where it strikes.
-[Weapon | Range: Mid | Delay: E+ (2.45x) | Slots: 4]
+[Weapon | Range: Mid | Delay: E+ (2.05x) | Slots: 4]
 Innate: Fire Magic +15% | Normal attacks: Paralysis chance (20%) | Phys Hit +10%</t>
         </is>
       </c>
@@ -10833,7 +10833,7 @@
       <c r="F281" t="inlineStr">
         <is>
           <t>You know the warden is a sadist when he pulls out the second whip.
-[Weapon | Range: Mid | Delay: D+ (2.15x) | Slots: 4]
+[Weapon | Range: Mid | Delay: D+ (1.85x) | Slots: 4]
 Innate: DEF +10% | Phys Hit +10% | Stab Res +50 | Aggro/Enmity +25%</t>
         </is>
       </c>
@@ -10870,7 +10870,7 @@
       <c r="F282" t="inlineStr">
         <is>
           <t>Cursed whip that grants an all-too-pleasant death.
-[Weapon | Range: Mid | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Mid | Delay: D (1.95x) | Slots: 4]
 Innate: Water Magic +15% | DEF +10% | Water Res +20</t>
         </is>
       </c>
@@ -10907,7 +10907,7 @@
       <c r="F283" t="inlineStr">
         <is>
           <t>Highly dangerous whip that exploits nuclear energy.
-[Weapon | Range: Mid | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Mid | Delay: D (1.95x) | Slots: 4]
 Innate: Physical ATK vs. Magic Beings +50% | DEF +10% | Crit Rate +10%</t>
         </is>
       </c>
@@ -10944,7 +10944,7 @@
       <c r="F284" t="inlineStr">
         <is>
           <t>Made of cords once used to restrain a wolf feared by the gods themselves.
-[Weapon | Range: Mid | Delay: E+ (2.45x) | Slots: 4]
+[Weapon | Range: Mid | Delay: E+ (2.05x) | Slots: 4]
 Innate: Physical ATK vs. Beasts +100% | Action Speed +10% | Nullify stun</t>
         </is>
       </c>
@@ -10981,7 +10981,7 @@
       <c r="F285" t="inlineStr">
         <is>
           <t>A pretty fan. Not only for attacks, but also defense.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 0]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 0]
 Innate: Standard equipment without innate passive enchantments.</t>
         </is>
       </c>
@@ -11018,7 +11018,7 @@
       <c r="F286" t="inlineStr">
         <is>
           <t>Statement fan for the newly rich. Those bills almost look real.
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 4]
 Innate: Aggro/Enmity +25% | Aggro/Enmity +25% | Aggro/Enmity +25% | Aggro/Enmity +25%</t>
         </is>
       </c>
@@ -11055,7 +11055,7 @@
       <c r="F287" t="inlineStr">
         <is>
           <t>Combat harisen that hits a bit too hard for comedy.
-[Weapon | Range: Short | Delay: D+ (2.15x) | Slots: 2]
+[Weapon | Range: Short | Delay: D+ (1.85x) | Slots: 2]
 Innate: Normal attacks: Silence chance (20%) | All Phys Res +15</t>
         </is>
       </c>
@@ -11092,7 +11092,7 @@
       <c r="F288" t="inlineStr">
         <is>
           <t>Wave it to kick up a cool breeze. For those hot summer nights.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 3]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 3]
 Innate: Wind Magic +15% | Magic DEF +10% | Action Speed +10%</t>
         </is>
       </c>
@@ -11129,7 +11129,7 @@
       <c r="F289" t="inlineStr">
         <is>
           <t>A fan made of the feathers of the legendary thunderbird.
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 4]
 Innate: Lightning Magic +15% | DEX +10% | Interrupt Rate -50% | Lightning Res +20</t>
         </is>
       </c>
@@ -11166,7 +11166,7 @@
       <c r="F290" t="inlineStr">
         <is>
           <t>Waft, strike--your choice. Has odd grooves that could retain liquid...
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 4]
 Innate: Normal attacks: Poison chance (20%) | AGI +10% | Phys Dodge +10%</t>
         </is>
       </c>
@@ -11203,7 +11203,7 @@
       <c r="F291" t="inlineStr">
         <is>
           <t>Make one dumb remark and you'll get hit.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 3]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 3]
 Innate: Phys ATK +10% | HP Regen +2%/turn | Slash Res +50</t>
         </is>
       </c>
@@ -11240,7 +11240,7 @@
       <c r="F292" t="inlineStr">
         <is>
           <t>Big fan wrought of holy silver. You feel holier just looking at it.
-[Weapon | Range: Short | Delay: D+ (2.15x) | Slots: 3]
+[Weapon | Range: Short | Delay: D+ (1.85x) | Slots: 3]
 Innate: Physical ATK vs. Demons +20% | Physical ATK vs. Undead +20% | Wind Res +50</t>
         </is>
       </c>
@@ -11277,7 +11277,7 @@
       <c r="F293" t="inlineStr">
         <is>
           <t>Beautiful and elegant fan. A lovely accent to a traditional dance.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 4]
 Innate: Action Speed +10% | Interrupt Rate -50% | Magic Damage Taken -10%</t>
         </is>
       </c>
@@ -11314,7 +11314,7 @@
       <c r="F294" t="inlineStr">
         <is>
           <t>Person-sized fan that can play the wind like a harp.
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 4]
 Innate: Wind Magic +15% | AGI +5% | Action Speed +10% | Wind Res +20</t>
         </is>
       </c>
@@ -11351,7 +11351,7 @@
       <c r="F295" t="inlineStr">
         <is>
           <t>An eardrum-shattering roar will echo throughout the galaxy.
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 4]
 Innate: Action Speed +10% | Phys Damage Taken -10% | Doll Potency +10%</t>
         </is>
       </c>
@@ -11388,7 +11388,7 @@
       <c r="F296" t="inlineStr">
         <is>
           <t>Historic fan of great significance in a southern kingdom.
-[Weapon | Range: Short | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Short | Delay: D (1.95x) | Slots: 4]
 Innate: Normal attacks: Sleep chance (20%) | Action Speed +10%</t>
         </is>
       </c>
@@ -11425,7 +11425,7 @@
       <c r="F297" t="inlineStr">
         <is>
           <t>Fan that can blow boulders away with just one wave.
-[Weapon | Range: Short | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Short | Delay: C+ (1.60x) | Slots: 4]
 Innate: Wind Magic +15% | Phys ATK +10% | Crit Rate +10% | Action Speed +10%</t>
         </is>
       </c>
@@ -11462,7 +11462,7 @@
       <c r="F298" t="inlineStr">
         <is>
           <t>Enchanted fan that turns a light waft into a chilling gust.
-[Weapon | Range: Short | Delay: D (2.3x) | Slots: 4]
+[Weapon | Range: Short | Delay: D (1.95x) | Slots: 4]
 Innate: Water Magic +15% | Earth Res +50 | Doll Potency +10%</t>
         </is>
       </c>
@@ -11499,7 +11499,7 @@
       <c r="F299" t="inlineStr">
         <is>
           <t>Golden fan borrowed from a hero who borrows the power of the sun.
-[Weapon | Range: Short | Delay: E+ (2.45x) | Slots: 4]
+[Weapon | Range: Short | Delay: E+ (2.05x) | Slots: 4]
 Innate: DEF +10% | Magic DEF +10% | Fire Res +50 | Nullify poison</t>
         </is>
       </c>
@@ -11536,7 +11536,7 @@
       <c r="F300" t="inlineStr">
         <is>
           <t>Symbol of a benevolent god who saved his people from the abyss.
-[Weapon | Range: Short | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Short | Delay: C (1.75x) | Slots: 4]
 Innate: All Elem Res +15 | TP Regen +6/turn | Double EXP</t>
         </is>
       </c>
@@ -11573,7 +11573,7 @@
       <c r="F301" t="inlineStr">
         <is>
           <t>Cheap, plastic megaphone.
-[Weapon | Range: Mid | Delay: B (1.6x) | Slots: 2]
+[Weapon | Range: Mid | Delay: B (1.45x) | Slots: 2]
 Innate: Aggro/Enmity -25% | Interrupt Rate -25%</t>
         </is>
       </c>
@@ -11610,7 +11610,7 @@
       <c r="F302" t="inlineStr">
         <is>
           <t>Mic that sweetens your voice and makes you a good talker.
-[Weapon | Range: Mid | Delay: C+ (1.8x) | Slots: 3]
+[Weapon | Range: Mid | Delay: C+ (1.60x) | Slots: 3]
 Innate: Max TP +5% | Phys Dodge +10% | Song Potency +10%</t>
         </is>
       </c>
@@ -11647,7 +11647,7 @@
       <c r="F303" t="inlineStr">
         <is>
           <t>As good for singing karaoke as for dishing sweet gossip.
-[Weapon | Range: Mid | Delay: C (2.0x) | Slots: 3]
+[Weapon | Range: Mid | Delay: C (1.75x) | Slots: 3]
 Innate: Phys DEF +10% | Magic DEF +10% | Chant Speed +15%</t>
         </is>
       </c>
@@ -11684,7 +11684,7 @@
       <c r="F304" t="inlineStr">
         <is>
           <t>Enhanced electric megaphone.
-[Weapon | Range: Mid | Delay: C (2.0x) | Slots: 3]
+[Weapon | Range: Mid | Delay: C (1.75x) | Slots: 3]
 Innate: Max HP +5% | Chant Speed +15% | Song Potency +10%</t>
         </is>
       </c>
@@ -11721,7 +11721,7 @@
       <c r="F305" t="inlineStr">
         <is>
           <t>Even a poor talker will be fine using this.
-[Weapon | Range: Mid | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Mid | Delay: B (1.45x) | Slots: 4]
 Innate: Aggro/Enmity -25% | Chant Speed +15% | Interrupt Rate -50%</t>
         </is>
       </c>
@@ -11758,7 +11758,7 @@
       <c r="F306" t="inlineStr">
         <is>
           <t>Disturbs its holder's sense of harmony, bringing pain to all who hear.
-[Weapon | Range: Mid | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Mid | Delay: C (1.75x) | Slots: 4]
 Innate: RES +10% | Interrupt Rate -90% | Phys Damage Taken -5%</t>
         </is>
       </c>
@@ -11795,7 +11795,7 @@
       <c r="F307" t="inlineStr">
         <is>
           <t>A legendary diva is said to have used this mic.
-[Weapon | Range: Mid | Delay: B+ (1.4x) | Slots: 3]
+[Weapon | Range: Mid | Delay: B+ (1.30x) | Slots: 3]
 Innate: Nullify silence | Chant Speed +15% | Song Potency +10%</t>
         </is>
       </c>
@@ -11832,7 +11832,7 @@
       <c r="F308" t="inlineStr">
         <is>
           <t>Emits a cursed wail that maddens those who hear it.
-[Weapon | Range: Mid | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Mid | Delay: B (1.45x) | Slots: 4]
 Innate: Normal attacks: Paralysis chance (20%) | Phys Dodge +10% | Magic Dodge +10%</t>
         </is>
       </c>
@@ -11869,7 +11869,7 @@
       <c r="F309" t="inlineStr">
         <is>
           <t>Can transmit an overbearing sound directly into an enemy's skull.
-[Weapon | Range: Mid | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Mid | Delay: C+ (1.60x) | Slots: 4]
 Innate: Normal attacks: Stun chance (20%) | Chant Speed +8% | Interrupt Rate -90%</t>
         </is>
       </c>
@@ -11906,7 +11906,7 @@
       <c r="F310" t="inlineStr">
         <is>
           <t>Magic mic that can change your voice into whatever you'd like.
-[Weapon | Range: Mid | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Mid | Delay: B (1.45x) | Slots: 4]
 Innate: Max TP +10% | Chant Speed +15% | TP Regen +4/turn | Song Potency +10%</t>
         </is>
       </c>
@@ -11943,7 +11943,7 @@
       <c r="F311" t="inlineStr">
         <is>
           <t>Mic that makes you spit fire.
-[Weapon | Range: Mid | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Mid | Delay: B+ (1.30x) | Slots: 4]
 Innate: Enemy Crit -10% | Interrupt Rate -90% | Song Potency +10%</t>
         </is>
       </c>
@@ -11980,7 +11980,7 @@
       <c r="F312" t="inlineStr">
         <is>
           <t>A legendary idol once used this mic.
-[Weapon | Range: Mid | Delay: A (1.2x) | Slots: 4]
+[Weapon | Range: Mid | Delay: A (1.15x) | Slots: 4]
 Innate: Phys Dodge +10% | Chant Speed +15% | Nullify silence | Song Potency +10%</t>
         </is>
       </c>
@@ -12017,7 +12017,7 @@
       <c r="F313" t="inlineStr">
         <is>
           <t>A mic oft used by the god of poetry.
-[Weapon | Range: Mid | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Mid | Delay: C+ (1.60x) | Slots: 4]
 Innate: Max TP +10% | RES +10% | Magic ATK +10% | Song Potency +10%</t>
         </is>
       </c>
@@ -12054,7 +12054,7 @@
       <c r="F314" t="inlineStr">
         <is>
           <t>Orders spoken through this mic are irresistible and must be obeyed.
-[Weapon | Range: Mid | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Mid | Delay: B (1.45x) | Slots: 4]
 Innate: Damage Taken -10% | Song Potency +20% (Carol/Chorale etc.) | TP Regen +4/turn</t>
         </is>
       </c>
@@ -12091,7 +12091,7 @@
       <c r="F315" t="inlineStr">
         <is>
           <t>The song slips into your heart and destroys your spirit.
-[Weapon | Range: Mid | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Mid | Delay: B+ (1.30x) | Slots: 4]
 Innate: Normal attacks: High Instakill chance (50%)</t>
         </is>
       </c>
@@ -12128,7 +12128,7 @@
       <c r="F316" t="inlineStr">
         <is>
           <t>Between the notes you can hear the trundling of a ramen cart.
-[Weapon | Range: Mid | Delay: C+ (1.8x) | Slots: 2]
+[Weapon | Range: Mid | Delay: C+ (1.60x) | Slots: 2]
 Innate: Max HP +5% | Action Speed +10%</t>
         </is>
       </c>
@@ -12165,7 +12165,7 @@
       <c r="F317" t="inlineStr">
         <is>
           <t>Repel evil spirits. A shrine maiden's best friend.
-[Weapon | Range: Mid | Delay: C (2.0x) | Slots: 2]
+[Weapon | Range: Mid | Delay: C (1.75x) | Slots: 2]
 Innate: AGI +10% | Dance Potency +10%</t>
         </is>
       </c>
@@ -12202,7 +12202,7 @@
       <c r="F318" t="inlineStr">
         <is>
           <t>The forbidden recorder. You must not give in to temptation.
-[Weapon | Range: Mid | Delay: C (2.0x) | Slots: 3]
+[Weapon | Range: Mid | Delay: C (1.75x) | Slots: 3]
 Innate: DEF +10% | Interrupt Rate -50% | HP Regen +4%/turn</t>
         </is>
       </c>
@@ -12239,7 +12239,7 @@
       <c r="F319" t="inlineStr">
         <is>
           <t>Bells employed by Uzume during the infamous dancing incident.
-[Weapon | Range: Mid | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Mid | Delay: C+ (1.60x) | Slots: 4]
 Innate: DEX +10% | Phys Dodge +10% | Enemy Crit -10% | Dance Potency +10%</t>
         </is>
       </c>
@@ -12276,7 +12276,7 @@
       <c r="F320" t="inlineStr">
         <is>
           <t>Simple instrument played with a snap of the wrist. Yosakoi!
-[Weapon | Range: Mid | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Mid | Delay: B (1.45x) | Slots: 4]
 Innate: Action Speed +10% | Interrupt Rate -25% | Dance Potency +10%</t>
         </is>
       </c>
@@ -12313,7 +12313,7 @@
       <c r="F321" t="inlineStr">
         <is>
           <t>Harmonica of a wanderer who's friends with a troll.
-[Weapon | Range: Mid | Delay: C+ (1.8x) | Slots: 3]
+[Weapon | Range: Mid | Delay: C+ (1.60x) | Slots: 3]
 Innate: Magic DEF +10% | Magic Dodge +10% | Wind Res +50</t>
         </is>
       </c>
@@ -12350,7 +12350,7 @@
       <c r="F322" t="inlineStr">
         <is>
           <t>Shining euphonium with a mellow sound.
-[Weapon | Range: Mid | Delay: D+ (2.15x) | Slots: 4]
+[Weapon | Range: Mid | Delay: D+ (1.85x) | Slots: 4]
 Innate: Normal attacks: Stun chance (20%) | DEF +10% | Interrupt Rate -50%</t>
         </is>
       </c>
@@ -12387,7 +12387,7 @@
       <c r="F323" t="inlineStr">
         <is>
           <t>Makes you want to dress up in green and go out hunting triangles.
-[Weapon | Range: Mid | Delay: B+ (1.4x) | Slots: 4]
+[Weapon | Range: Mid | Delay: B+ (1.30x) | Slots: 4]
 Innate: Wind Magic +15% | Interrupt Rate -50% | Damage -&gt; TP (10%) | Wind Res +50</t>
         </is>
       </c>
@@ -12424,7 +12424,7 @@
       <c r="F324" t="inlineStr">
         <is>
           <t>A lefty bass with a sunburst finish. Quick, give it a nickname!
-[Weapon | Range: Mid | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Mid | Delay: C (1.75x) | Slots: 4]
 Innate: Interrupt Rate -90% | Magic Damage Taken -10% | All Phys Res +50</t>
         </is>
       </c>
@@ -12461,7 +12461,7 @@
       <c r="F325" t="inlineStr">
         <is>
           <t>Flute made from hollow water reeds that were once a nymph.
-[Weapon | Range: Mid | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Mid | Delay: C+ (1.60x) | Slots: 4]
 Innate: Normal attacks: Sleep chance (20%) | Action Speed +10% | Bash Res +50</t>
         </is>
       </c>
@@ -12498,7 +12498,7 @@
       <c r="F326" t="inlineStr">
         <is>
           <t>Let's jam out on three strings at the center of the world.
-[Weapon | Range: Mid | Delay: C (2.0x) | Slots: 4]
+[Weapon | Range: Mid | Delay: C (1.75x) | Slots: 4]
 Innate: AGI +10% | HP Regen +4%/turn | Dance Potency +10% | Nullify freeze</t>
         </is>
       </c>
@@ -12535,7 +12535,7 @@
       <c r="F327" t="inlineStr">
         <is>
           <t>Flute of the god of music. It gives off a nice sound.
-[Weapon | Range: Mid | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Mid | Delay: B (1.45x) | Slots: 4]
 Innate: DEF +10% | Interrupt Rate -90% | Dance Potency +10%</t>
         </is>
       </c>
@@ -12572,7 +12572,7 @@
       <c r="F328" t="inlineStr">
         <is>
           <t>Dastardly wind instrument that inspires hearts to evil.
-[Weapon | Range: Mid | Delay: C+ (1.8x) | Slots: 4]
+[Weapon | Range: Mid | Delay: C+ (1.60x) | Slots: 4]
 Innate: Physical ATK vs. Magic Beings +100% | Normal attacks: Paralysis chance (20%)</t>
         </is>
       </c>
@@ -12609,7 +12609,7 @@
       <c r="F329" t="inlineStr">
         <is>
           <t>Trumpet that signals the end. By the time you hear it, it's too late.
-[Weapon | Range: Mid | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Mid | Delay: B (1.45x) | Slots: 4]
 Innate: All stats +3 | Interrupt Rate -50% | All Phys Res +50 | Dance Potency +10%</t>
         </is>
       </c>
@@ -12646,7 +12646,7 @@
       <c r="F330" t="inlineStr">
         <is>
           <t>A goddess's stringed instrument. It takes four arms to play...
-[Weapon | Range: Mid | Delay: B (1.6x) | Slots: 4]
+[Weapon | Range: Mid | Delay: B (1.45x) | Slots: 4]
 Innate: DEF +10% | Interrupt Rate -90% | All Elem Res +50 | Dance Potency +20%</t>
         </is>
       </c>

</xml_diff>

<commit_message>
feat: implement JP community QoL improvements - Smooth EXP curve
implement JP community QoL improvements - Smooth EXP curve, Catch- up
Double EXP training gear, and Grand Seal EXP parity
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/equipment.xlsx
+++ b/mod_project/data_tables/equipment.xlsx
@@ -19448,14 +19448,14 @@
       </c>
       <c r="E514" t="inlineStr">
         <is>
-          <t>In fact a heavy shackle, broken free of its chain.</t>
+          <t>In fact a heavy training shackle, broken free of its chain.</t>
         </is>
       </c>
       <c r="F514" t="inlineStr">
         <is>
-          <t>In fact a heavy shackle, broken free of its chain.
+          <t>In fact a heavy training shackle, broken free of its chain.
 [Accessory | Slots: 3]
-Innate: AGI -10% | Phys Damage Taken -10% | Phys Damage Taken -10%</t>
+Innate: AGI -10% | Phys Damage Taken -10% | Double EXP</t>
         </is>
       </c>
       <c r="G514" t="inlineStr">

</xml_diff>